<commit_message>
BRD-02 Operations sign-off set v2.0 rebuilt on the final retake: Start Here, guide deck, FRS, sign-off workbook, test plan and summary; UX screen deck, UX screen register and image package; ACSL persona texts, the ACSL team leader's menu kept once; drop index
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-02_Operations/04_BIBS_TestPlan_BRD-02_Operations_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-02_Operations/04_BIBS_TestPlan_BRD-02_Operations_v2.0.xlsx
@@ -13503,7 +13503,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr"/>
@@ -13591,7 +13591,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>1. As mktcoll open Remittance Holds, Special Remittance and BIR 2307; open the waiting hold of ARN-2026-940004.</t>
+          <t>1. As mktcoll open Remittance Holds, Special Remittance and BIR 2307; open the waiting hold of ARN-2026-940008.</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
@@ -14110,7 +14110,7 @@
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr"/>
@@ -14269,13 +14269,13 @@
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>The hold of ARN-2026-940004 approved (TC-OP-111.1-01).
+          <t>The hold of ARN-2026-940008 approved (TC-OP-111.1-01).
 Data: TD-OP-02 Booked seed invoices; TD-OP-04 Remittance storyline</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>1. Open Invoice 360 of ARN-2026-940004, Remittances tab.</t>
+          <t>1. Open Invoice 360 of ARN-2026-940008, Remittances tab.</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
@@ -14509,7 +14509,7 @@
       <c r="L22" s="12" t="inlineStr">
         <is>
           <t>Refused.
-Message "Invoice &lt;no&gt; is locked by REMITTANCE (&lt;reason&gt;)" (INVOICE_LOCKED).</t>
+Message "Invoice &lt;no&gt; is locked by &lt;team&gt; (&lt;reason&gt;)" (INVOICE_LOCKED).</t>
         </is>
       </c>
       <c r="M22" s="12" t="inlineStr">
@@ -14580,7 +14580,7 @@
       </c>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>1. Receive a payment on the invoice of ARN-2026-940004 (open cancellation request, locked by ADJUSTMENT).</t>
+          <t>1. Receive a payment on the invoice of ARN-2026-940004 (open cancellation request, locked by Adjustment).</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr">
@@ -16386,7 +16386,7 @@
       </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I47" s="12" t="inlineStr"/>
@@ -16921,7 +16921,7 @@
       </c>
       <c r="H54" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I54" s="12" t="inlineStr"/>
@@ -19825,7 +19825,7 @@
       </c>
       <c r="L92" s="12" t="inlineStr">
         <is>
-          <t>None is offered; BIBS refuses any change.</t>
+          <t>None is offered; an attempt to change an entry outside the screens is refused.</t>
         </is>
       </c>
       <c r="M92" s="12" t="inlineStr">
@@ -20034,7 +20034,7 @@
       </c>
       <c r="H95" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I95" s="12" t="inlineStr"/>
@@ -20565,7 +20565,7 @@
       </c>
       <c r="H102" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I102" s="12" t="inlineStr"/>
@@ -20791,7 +20791,7 @@
       </c>
       <c r="H105" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I105" s="12" t="inlineStr"/>
@@ -20947,13 +20947,13 @@
       </c>
       <c r="J107" s="12" t="inlineStr">
         <is>
-          <t>The hold of ARN-2026-940004 approved.
+          <t>The hold of ARN-2026-940008 approved.
 Data: TD-OP-02 Booked seed invoices; TD-OP-04 Remittance storyline</t>
         </is>
       </c>
       <c r="K107" s="12" t="inlineStr">
         <is>
-          <t>1. Run the extraction; open the tag of ARN-2026-940004.</t>
+          <t>1. Run the extraction; open the tag of ARN-2026-940008.</t>
         </is>
       </c>
       <c r="L107" s="12" t="inlineStr">
@@ -21618,7 +21618,7 @@
       </c>
       <c r="H116" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I116" s="12" t="inlineStr"/>
@@ -23601,7 +23601,7 @@
       </c>
       <c r="H142" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I142" s="12" t="inlineStr"/>
@@ -24056,7 +24056,7 @@
       </c>
       <c r="H148" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I148" s="12" t="inlineStr"/>
@@ -25125,7 +25125,7 @@
       </c>
       <c r="H162" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I162" s="12" t="inlineStr"/>
@@ -27315,7 +27315,7 @@
       </c>
       <c r="H191" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I191" s="12" t="inlineStr"/>
@@ -28378,7 +28378,7 @@
       </c>
       <c r="H205" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I205" s="12" t="inlineStr"/>
@@ -28910,7 +28910,7 @@
       </c>
       <c r="H212" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I212" s="12" t="inlineStr"/>
@@ -29974,7 +29974,7 @@
       </c>
       <c r="H226" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I226" s="12" t="inlineStr"/>
@@ -31059,7 +31059,7 @@
       <c r="L240" s="12" t="inlineStr">
         <is>
           <t>The row is refused.
-Message "Decision '&lt;value&gt;' is neither APPROVED nor REJECTED" (DP_RESPONSE_DECISION).</t>
+Message "Decision '&lt;value&gt;' is not one of Approved or Rejected (or Yes / No)" (DP_RESPONSE_DECISION).</t>
         </is>
       </c>
       <c r="M240" s="12" t="inlineStr">
@@ -31594,7 +31594,7 @@
       <c r="L247" s="12" t="inlineStr">
         <is>
           <t>Refused.
-Message "Scheme &lt;name&gt; has no tiers yet (targets and amounts from BDOI, OQ39)" (INCENTIVE_SCHEME_EMPTY).</t>
+Message "Scheme &lt;name&gt; has no tiers yet: add its targets and amounts first" (INCENTIVE_SCHEME_EMPTY).</t>
         </is>
       </c>
       <c r="M247" s="12" t="inlineStr">
@@ -32261,7 +32261,7 @@
       </c>
       <c r="H256" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I256" s="12" t="inlineStr"/>
@@ -32579,7 +32579,7 @@
       </c>
       <c r="K260" s="12" t="inlineStr">
         <is>
-          <t>1. As mkttl open the waiting hold of ARN-2026-940004; Approve hold; as remit run the extraction.</t>
+          <t>1. As mkttl open the waiting hold of ARN-2026-940008; Approve hold; as remit run the extraction.</t>
         </is>
       </c>
       <c r="L260" s="12" t="inlineStr">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="K263" s="12" t="inlineStr">
         <is>
-          <t>1. Request a hold on ARN-2026-940004 again.</t>
+          <t>1. Request a hold on ARN-2026-940008 again.</t>
         </is>
       </c>
       <c r="L263" s="12" t="inlineStr">
@@ -33789,7 +33789,7 @@
       </c>
       <c r="H276" s="12" t="inlineStr">
         <is>
-          <t>Access check outside the screens, run by the test lead signed in as the persona</t>
+          <t>System function check outside the screens, signed in as the persona (test lead tool)</t>
         </is>
       </c>
       <c r="I276" s="12" t="inlineStr"/>
@@ -34724,7 +34724,7 @@
       <c r="L288" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-02 Invoice Search of the FRS.
-Fields in this order: 1 All Invoices / Outstanding / Paid, Not Extracted / On Hold / Locked / Direct Payment (Tab, mandatory -); 2 Search Invoice No., ARN, policy, client or assured (Text, mandatory N); 3 Origin (Drop-down, mandatory N); 4 Insurer Code / Name of Assured / Account Officer (Text, mandatory N); 5 Booked From / Booked To / Inception From / Inception To (Date, mandatory N); 6 Invoice No. (Column, mandatory -); 7 Assured / Client Code (Column, mandatory -); 8 Insurer (Column, mandatory -); 9 Booked / Inception (Column, mandatory -); 10 Account Officer (Column, mandatory -); 11 Gross Premium / Outstanding (Column, mandatory -); 12 Status / Remittance (Column, mandatory -); 13 Flags (Column, mandatory -).
+Fields in this order: 1 All Invoices / Outstanding / Paid, Not Extracted / On Hold / Locked / Direct Payment (Tab, mandatory -); 2 Search Invoice No., ARN, policy, client or assured (Text, mandatory N); 3 Origin (Drop-down, mandatory N); 4 Insurer / Name of Assured / Account Officer (Drop-down, text, mandatory N); 5 Booked From / Booked To / Inception From / Inception To (Date, mandatory N); 6 Invoice No. (Column, mandatory -); 7 Assured / Client Code (Column, mandatory -); 8 Insurer (Column, mandatory -); 9 Booked / Inception (Column, mandatory -); 10 Account Officer (Column, mandatory -); 11 Gross Premium / Outstanding (Column, mandatory -); 12 Status / Remittance (Column, mandatory -); 13 Flags (Column, mandatory -).
 Actions: Search; Filters / Apply Filters; Open a row.</t>
         </is>
       </c>
@@ -34802,7 +34802,7 @@
       <c r="L289" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-03 Invoice 360 of the FRS.
-Fields in this order: 1 Invoice / ARN / Policy No. / Endorsement / Root Invoice (Reference chip, mandatory -); 2 Payment status and remittance status pills (Status pill, mandatory -); 3 Flags (Tag, mandatory -); 4 Client / Insurer(s) / Period / Gross / Outstanding Premium / Booked (Display, mandatory -); 5 Account workflow header (Stepper, mandatory -); 6 Components &amp; Balances / Movements / Invoice Family / Policy Transactions / Receipts / Remittances / Adjustments / Reconciliation / Commission / History / Documents (Tab, mandatory -); 7 Component / Booked / Applied / Reversed / Remitted / Adjusted / Written Off / Balance (Column, mandatory -); 8 Premium Due / Premium Collected / Premium Outstanding (Display, mandatory -); 9 Insurer Shares (Table, mandatory -); 10 Value Date / Movement / Component / Amount / Source / Documents / Posted (Column, mandatory -); 11 Invoice No. / Transaction / Booked / Gross Premium / Outstanding / Payment / Remittance (Column, mandatory -); 12 Date / Transaction / Reference / Premium Change / Taxes Change / Commission Change / Gross Premium After / Status / Accounting (Column, mandatory -); 13 GL Account / Party / Narration / Debit / Credit (Column, mandatory -); 14 Record / Reference / Date / Amount / Status / Description (Column, mandatory -); 15 When / What / Change / Module / Reason / By (Column, mandatory -); 16 Documents panel (Panel, mandatory -).
+Fields in this order: 1 Invoice / ARN / Policy No. / Endorsement / Root Invoice (Reference chip, mandatory -); 2 Payment status and remittance status pills (Status pill, mandatory -); 3 Flags (Tag, mandatory -); 4 Client / Insurer(s) / Period / Gross / Outstanding Premium / Booked (Display, mandatory -); 5 Account workflow header (Stepper, mandatory -); 6 Components &amp; Balances / Movements / Invoice Family / Policy Transactions / Receipts / Remittances / Adjustments / Reconciliation / Commission / History / Documents (Tab, mandatory -); 7 Component / Booked / Applied / Reversed / Remitted / Adjusted / Written Off / Balance (Column, mandatory -); 8 Premium Due / Premium Collected / Premium Outstanding (Display, mandatory -); 9 Insurer Shares (Table, mandatory -); 10 Value Date / Movement / Component / Amount / Source / Documents / Posted (Column, mandatory -); 11 Invoice No. / Transaction / Booked / Gross Premium / Outstanding / Payment / Remittance (Column, mandatory -); 12 Date / Transaction / Reference / Premium Change / Taxes / Commission / Gross Premium After / Status / Accounting (Column, mandatory -); 13 GL Account / Party / Narration / Debit / Credit (Column, mandatory -); 14 Record / Reference / Date / Amount / Status / Description (Column, mandatory -); 15 When / What / Change / Module / Reason / By (Column, mandatory -); 16 Documents panel (Panel, mandatory -).
 Actions: Open Booked Invoice; A reference in a tab; Journals button of a Policy Transactions row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -34882,7 +34882,7 @@
         <is>
           <t>The screen matches SCR-OP-04 Hand-offs and Extracts of the FRS.
 Fields in this order: 1 Open Hand-offs / Closed Hand-offs / Extract Repository (Tab, mandatory -); 2 Work / What To Do / From / Amount / Created / Status (Column, mandatory -); 3 What Was Done (Text, mandatory Y); 4 Folder / File / From / Size / Stored (Column, mandatory -); 5 Download (Button, mandatory -).
-Actions: Close; Download.
+Actions: Close Hand-off; Download.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -34959,7 +34959,7 @@
       <c r="L291" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-05 Report Archive of the FRS.
-Fields in this order: 1 Search Report Code, e.g. CSH-APPLIED-PREM (Text, mandatory N); 2 Report (Column, mandatory -); 3 Parameters (Column, mandatory -); 4 Action (Column, mandatory -); 5 Rows (Column, mandatory -); 6 Generated (Column, mandatory -); 7 File (Column, mandatory -).
+Fields in this order: 1 Report (Drop-down, mandatory N); 2 Report (Column, mandatory -); 3 Parameters (Column, mandatory -); 4 Action (Column, mandatory -); 5 Rows (Column, mandatory -); 6 Generated (Column, mandatory -); 7 File (Column, mandatory -).
 Actions: Search; Download.</t>
         </is>
       </c>
@@ -35270,7 +35270,7 @@
       <c r="L295" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-09 Receipts of the FRS.
-Fields in this order: 1 Receipts / Cancellations and Reinstatements (Tab, mandatory -); 2 Search Receipt No. (Text, mandatory N); 3 Client Code / Invoice No. / Policy No. / Payor Name / Assured Name / Insurer Code (Text, mandatory N); 4 Amount / Date From / Date To (Number, Date, mandatory N); 5 Kind / Status (Drop-down, mandatory N); 6 Receipt No. / Date / Payor / Assured / Mode / Amount / Applied / Unapplied / Status (Column, mandatory -); 7 Transaction No. / Reason / Amount / Requested / Status (Column, mandatory -); 8 OR Type (Drop-down, mandatory Y); 9 Payor Name / Payor Code (Text, mandatory Y / N); 10 Currency / Mode of Payment / Check No. (Text, Drop-down, mandatory Y / N / N); 11 Gross Amount / VAT / Withholding Tax (Number, mandatory Y / N / N); 12 2307 Certificate Ref. / Description (Text, mandatory N).
+Fields in this order: 1 Receipts / Cancellations and Reinstatements (Tab, mandatory -); 2 Search Receipt No. (Text, mandatory N); 3 Client Code / Invoice No. / Policy No. / Payor Name / Assured Name / Insurer (Text, drop-down, mandatory N); 4 Amount / Date From / Date To (Number, Date, mandatory N); 5 Kind / Status (Drop-down, mandatory N); 6 Receipt No. / Date / Payor / Assured / Mode / Amount / Applied / Unapplied / Status (Column, mandatory -); 7 Transaction No. / Reason / Amount / Requested / Status (Column, mandatory -); 8 OR Type (Drop-down, mandatory Y); 9 Payor Name / Payor Code (Text, mandatory Y / N); 10 Currency / Mode of Payment / Check No. (Text, Drop-down, mandatory Y / N / N); 11 Gross Amount / VAT / Withholding Tax (Number, mandatory Y / N / N); 12 2307 Certificate Ref. / Description (Text, mandatory N).
 Actions: Issue Official Receipt / Issue OR; Search / Filters; Open Receipt; Approve; Resubmit.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -35350,7 +35350,7 @@
         <is>
           <t>The screen matches SCR-OP-10 Receipt of the FRS.
 Fields in this order: 1 Receipt No. chip and status pill (Reference chip, status pill, mandatory -); 2 Flags (Tag, mandatory -); 3 Receipt Date / Payor / Amount / Applied / Unapplied / Mode / Currency / BOOK Rate (Display, mandatory -); 4 Receipt action workflow header (Stepper, mandatory -); 5 Applications / Lines / Journal / History (Tab, mandatory -); 6 Invoice / Reference / By Component / Applied / Commission Realized / Value Date / Status (Column, mandatory -); 7 Invoice / Item / Insurer / Gross / VAT / WTAX / Net (Column, mandatory -); 8 Journal Batch / Posting (Column, mandatory -); 9 Transaction No. / Action / Reason / Amount / Requested / Approved / Status (Column, mandatory -); 10 Reason (Drop-down, mandatory Y); 11 Comment (Text area, mandatory Cond.); 12 Full / Partial (Radio, mandatory Y); 13 Reason Group / Reason (Drop-down, mandatory Y); 14 Amount to Reinstate (Number, mandatory Cond.: partial); 15 Invoice No. / AR / OR No. / Assured / Payor / Account Officer / Unit Head / Team Leader / Remarks (Text, mandatory Y (Remarks N)).
-Actions: Print; Cancel Receipt; Reinstate; Approve and Post; Return to Requester.
+Actions: Print (PDF); Cancel Receipt; Reinstate; Approve and Post; Return to Requester.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -35507,7 +35507,7 @@
       <c r="L298" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-12 Unapplied Payment of the FRS.
-Fields in this order: 1 Reference chip, origin tag and stage pill (Reference chip, tag, status pill, mandatory -); 2 Amount / Balance / Payor / Client / Unit / Source / Received (Display, mandatory -); 3 Disposition workflow header (Stepper, mandatory -); 4 Disposition Type (Drop-down, mandatory Y); 5 Amount (Number, mandatory Y); 6 Apply to Invoice No. / Reclass to Client Code / Transfer to Marketing Unit / Refund Payee (Text, mandatory Cond.); 7 Remarks (Text area, mandatory N); 8 Disposition / Amount / Target / Requested / Approved / Document / Status (Column, mandatory -); 9 Reason / Comment (Drop-down, text area, mandatory Y / N).
+Fields in this order: 1 Reference chip, origin tag and stage pill (Reference chip, tag, status pill, mandatory -); 2 Amount / Balance / Payor / Marketing Unit / Source / Received (Display, mandatory -); 3 Disposition workflow header (Stepper, mandatory -); 4 Disposition Type (Drop-down, mandatory Y); 5 Amount (Number, mandatory Y); 6 Apply to Invoice No. / Reclass to Client Code / Transfer to Marketing Unit / Refund Payee (Text, mandatory Cond.); 7 Remarks (Text area, mandatory N); 8 Disposition / Amount / Target / Requested / Approved / Document / Status (Column, mandatory -); 9 Reason / Comment (Drop-down, text area, mandatory Y / N).
 Actions: Save Disposition; Submit for Approval; Process Disposition; Approve; Return to Cashier; Withdraw Disposition; Mark for Reversal / Approve Reversal; Open Receipt.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -35666,7 +35666,7 @@
         <is>
           <t>The screen matches SCR-OP-14 Pre-booked Payments of the FRS.
 Fields in this order: 1 Waiting for Booking / Applied / Released to Unapplied (Tab, mandatory -); 2 Account (ARN) / Reference / Amount / Received / Age / Re-match Attempts / Receipt / Status (Column, mandatory -); 3 Comment (Text area, mandatory N).
-Actions: Run Matching Now; Re-match Now; Release.
+Actions: Run Matching Now; Open Receipt; Re-match Now; Release to Unapplied.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -35903,7 +35903,7 @@
         <is>
           <t>The screen matches SCR-OP-17 Check Pick-up of the FRS.
 Fields in this order: 1 For Pick-up / AR Printed / Cancelled (Tab, mandatory -); 2 Pick-up From / Pick-up To (Date, mandatory N); 3 Select (Check box, mandatory N); 4 Collection Ref. / Payor / Pick-up Date / Requested By / Check No. / Amount / AR / Status (Column, mandatory -).
-Actions: Import Pending Requests; Print ARs; Download &lt;batch&gt;; Cancel.
+Actions: Import Pending Requests; Print ARs; Download &lt;batch&gt;; Cancel Check Pick-up.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -35981,7 +35981,7 @@
       <c r="L304" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-18 Batch Print of the FRS.
-Fields in this order: 1 Kind / Insurer Code / Date From / Date To (Drop-down, text, date, mandatory N); 2 Receipt No. / Date / Payor / Amount / Printed (Column, mandatory -); 3 Batch No. / Criteria / Progress / Printed / Failed / Created / Status (Column, mandatory -).
+Fields in this order: 1 Kind / Insurer / Date From / Date To (Drop-down, date, mandatory N); 2 Receipt No. / Date / Payor / Amount / Printed (Column, mandatory -); 3 Batch No. / Criteria / Progress / Printed / Failed / Created / Status (Column, mandatory -).
 Actions: Preview List; Print Selected (n); Download; Retry Failures.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -36060,7 +36060,7 @@
       <c r="L305" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-19 BIR 2307 of the FRS.
-Fields in this order: 1 Tagged by Marketing / Validation / Reports and Routing / Released / Settled (Tab, mandatory -); 2 Reference / Client / Insurer / Path / Amount / Checklist / Tagged / Stage (Column, mandatory -); 3 CWT copy received (Check box, mandatory N); 4 Batch No. / Insurer / Certificates / Total / Disbursement / Status (Column, mandatory -); 5 Invoice No. (Text, mandatory Y); 6 Path (Drop-down, mandatory Y); 7 Amount (Number, mandatory N); 8 Certificate No. / Period From / Period To / Remarks (Text, date, mandatory Cond.).
+Fields in this order: 1 Tagged by Marketing / Validation / Reports and Routing / Released / Settled (Tab, mandatory -); 2 Reference / Client / Insurer / Path / Amount / Checklist / Tagged / Stage (Column, mandatory -); 3 CWT Copy Received (Row action (Mark / Clear CWT Copy Received), mandatory N); 4 Batch No. / Insurer / Certificates / Total / Disbursement / Status (Column, mandatory -); 5 Invoice No. (Text, mandatory Y); 6 Path (Drop-down, mandatory Y); 7 Amount (Number, mandatory N); 8 Certificate No. / Period From / Period To / Remarks (Text, date, mandatory Cond.).
 Actions: Tag 2307; Receive; Validate and Post Report; Settle in Cash; Route to Disbursement; Release to Insurer; Return to Marketing / Cancel Tag.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -36296,8 +36296,8 @@
       <c r="L308" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-22 Cashiering Setup of the FRS.
-Fields in this order: 1 Payment File Layouts / Minimal Balance (Tab, mandatory -); 2 File / Kind / Separator / Last Changed (Column, mandatory -); 3 File Kind / Separator / Fields (Header:start:length separated by ;, start is 1-based) (Drop-down, text, mandatory Y); 4 Balance / Up To / Excludes / Action / Status (Column, mandatory -).
-Actions: Edit / Save Layout; Run Sweep Now.</t>
+Fields in this order: 1 Payment File Layouts / Minimal Balance (Tab, mandatory -); 2 File / Kind / Separator / Last Changed (Column, mandatory -); 3 Fields / Separator / Fields (Header:start:length separated by ;, start is 1-based) (Drop-down, text, mandatory Y); 4 Balance / Up To / Excludes / Action / Status (Column, mandatory -).
+Actions: Edit Layout / Save Layout; Run Sweep Now.</t>
         </is>
       </c>
       <c r="M308" s="12" t="inlineStr">
@@ -36451,7 +36451,7 @@
       <c r="L310" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-24 Extraction of the FRS.
-Fields in this order: 1 Insurer Code (Text, mandatory N); 2 Remittance Type (Drop-down, mandatory N); 3 Invoice No. (Text, mandatory N); 4 Run No. / Scope / Status / Examined / Extracted / Due, Not Extracted / Not Yet Due / Batches / Started (Column, mandatory -); 5 Invoice No. / Insurer / Type / Tag / Reasons / Paid AR / Remitted Now / Batch (Column, mandatory -).
+Fields in this order: 1 Insurer (Drop-down, mandatory N); 2 Remittance Type (Drop-down, mandatory N); 3 Invoice No. (Text, mandatory N); 4 Run No. / Scope / Status / Examined / Extracted / Due, Not Extracted / Not Yet Due / Batches / Started (Column, mandatory -); 5 Invoice No. / Insurer / Type / Tag / Reasons / Paid AR / Remitted Now / Batch (Column, mandatory -).
 Actions: Run Extraction; Open a run.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -36530,7 +36530,7 @@
       <c r="L311" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-25 Remittance Batches of the FRS.
-Fields in this order: 1 Review in Process / For Approval / With Disbursement / Awaiting Insurer OR / OR Received / Returned (Tab, mandatory -); 2 Search Batch or Invoice No. (Text, mandatory N); 3 Insurer Code / Remittance Type (Text, drop-down, mandatory N); 4 Select (Check box, mandatory N); 5 Batch No. / Insurer / Type / Accounts / Paid AR / Payable / Currency / Processor / DV No. / Status (Column, mandatory -).
+Fields in this order: 1 Review in Process / For Approval / With Disbursement / Awaiting Insurer OR / OR Received / Returned (Tab, mandatory -); 2 Search Batch or Invoice No. (Text, mandatory N); 3 Insurer / Remittance Type (Drop-down, mandatory N); 4 Select (Check box, mandatory N); 5 Batch No. / Insurer / Type / Accounts / Paid AR / Payable / Currency / Processor / DV No. / Status (Column, mandatory -).
 Actions: Submit Selected; Approve Selected; Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -36688,7 +36688,7 @@
       <c r="L313" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-27 Insurer OR Upload of the FRS.
-Fields in this order: 1 Download Template (Button, mandatory -); 2 Insurer schedule file (File, mandatory Y); 3 Upload Run / File / Status / Accepted / Failed / Uploaded (Column, mandatory -); 4 Records Read / OR Matches Paid PR / Amount Mismatch / Refused (Tile, mandatory -); 5 Batch No. / Invoice No. / OR No. / OR Date / OR Amount / Paid PR / Status (Column, mandatory -); 6 Record / Result / Reason (Column, mandatory -).
+Fields in this order: 1 Download Template (Button, mandatory -); 2 Insurer Schedule (File, mandatory Y); 3 Upload Run / File / Status / Accepted / Failed / Uploaded (Column, mandatory -); 4 Records Read / OR Matches Paid PR / Amount Mismatch / Refused (Tile, mandatory -); 5 Batch No. / Invoice No. / OR No. / OR Date / OR Amount / Paid PR / Status (Column, mandatory -); 6 Record / Result / Reason (Column, mandatory -).
 Actions: Upload File; Open a run.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -36767,7 +36767,7 @@
       <c r="L314" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-28 Remittance Holds of the FRS.
-Fields in this order: 1 For Approval / Active Holds / Drafts / Released and Closed (Tab, mandatory -); 2 Search Hold or Invoice No. (Text, mandatory N); 3 Hold No. / Invoice No. / Name of Assured / Insurer / Reason / Hold Until / Processor / Status (Column, mandatory -); 4 Invoice No. (Text, mandatory Y); 5 Reason (Drop-down, mandatory Y); 6 Hold Until (Date, mandatory Y); 7 Remarks (Text area, mandatory N); 8 Hold file (File, mandatory Y).
+Fields in this order: 1 For Approval / Active Holds / Drafts / Released and Closed (Tab, mandatory -); 2 Search Hold or Invoice No. (Text, mandatory N); 3 Hold No. / Invoice No. / Name of Assured / Insurer / Reason / Hold Until / Processor / Status (Column, mandatory -); 4 Invoice No. (Text, mandatory Y); 5 Reason (Drop-down, mandatory Y); 6 Hold Until (Date, mandatory Y); 7 Remarks (Text area, mandatory N); 8 Hold File (File, mandatory Y).
 Actions: New Hold Request; Upload Hold File; Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -36846,7 +36846,7 @@
       <c r="L315" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-29 Remittance Hold of the FRS.
-Fields in this order: 1 Hold chip and stage pill (Reference chip, status pill, mandatory -); 2 Invoice / Insurer / Hold Until / Requested / Approved By / Processor (Display, mandatory -); 3 Hold workflow header (Stepper, mandatory -); 4 New Hold Until / Comment (Date, text, mandatory Y / N); 5 Remittance Processor (User ID) (Text, mandatory Y).
+Fields in this order: 1 Hold chip and stage pill (Reference chip, status pill, mandatory -); 2 Invoice / Insurer / Hold Until / Requested / Approved By / Processor (Display, mandatory -); 3 Hold workflow header (Stepper, mandatory -); 4 New Hold Until / Comment (Date, text, mandatory Y / N); 5 Remittance Processor (Drop-down, mandatory Y).
 Actions: Approve hold / Reject hold; Request extension / Approve extension / Reject extension; Request cancellation / Approve cancellation / Reject cancellation; Release hold; Assign to Processor.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -37082,7 +37082,7 @@
       <c r="L318" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-32 DTIP Status of the FRS.
-Fields in this order: 1 DTIP Status / Accounts in Batches (Tab, mandatory -); 2 Search Invoice, ARN, Policy or Assured (Text, mandatory N); 3 Insurer Code / Remittance Status (Text, drop-down, mandatory N); 4 Invoice No. / Insurer / Payment / Paid AR / DTIP / Remitted / Outstanding DTIP / Extraction Tag / Flags / Remittance Status (Column, mandatory -); 5 Batch No. / Invoice No. / Endorsement / Policy No. / Name of Assured / Paid AR / Net Due / Status (Column, mandatory -).
+Fields in this order: 1 DTIP Status / Accounts in Batches (Tab, mandatory -); 2 Search Invoice, ARN, Policy or Assured (Text, mandatory N); 3 Insurer / Remittance Status (Drop-down, mandatory N); 4 Invoice No. / Insurer / Payment / Paid AR / DTIP / Remitted / Outstanding DTIP / Extraction Tag / Flags / Remittance Status (Column, mandatory -); 5 Batch No. / Invoice No. / Endorsement / Policy No. / Name of Assured / Paid AR / Net Due / Status (Column, mandatory -).
 Actions: Queue for End of Day.</t>
         </is>
       </c>
@@ -37160,7 +37160,7 @@
       <c r="L319" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-33 Remittance Deductions of the FRS.
-Fields in this order: 1 For Confirmation / Confirmed / Drafts / Applied and Cancelled (Tab, mandatory -); 2 Search Deduction No. or Source Reference (Text, mandatory N); 3 Deduction No. / Insurer / Source / Insurer Confirmation / Amount / Remaining / Status (Column, mandatory -); 4 Insurer Code / Currency (Text, drop-down, mandatory Y); 5 Deduction Source / Source Reference / Invoice No. (Drop-down, text, mandatory Y / Y / N); 6 Amount (Number, mandatory Y); 7 Insurer Confirmation Ref. / Confirmation Date / Remarks (Text, date, mandatory N).
+Fields in this order: 1 For Confirmation / Confirmed / Drafts / Applied and Cancelled (Tab, mandatory -); 2 Search Deduction No. or Source Reference (Text, mandatory N); 3 Deduction No. / Insurer / Source / Insurer Confirmation / Amount / Remaining / Status (Column, mandatory -); 4 Insurer / Currency (Drop-down, mandatory Y); 5 Deduction Source / Source Reference / Invoice No. (Drop-down, text, mandatory Y / Y / N); 6 Amount (Number, mandatory Y); 7 Insurer Confirmation Ref. / Confirmation Date / Remarks (Text, date, mandatory N).
 Actions: New Deduction / Save Deduction; Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -37318,7 +37318,7 @@
       <c r="L321" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-35 Incentive Rules of the FRS.
-Fields in this order: 1 Insurer / Product Line / Segment / Rate / Window / Effective / Status (Column, mandatory -); 2 Insurer Code (Text, mandatory Y); 3 Product Line (blank = all) / Segment (blank = all) (Text, mandatory N); 4 Rate (% of basic premium) (Number, mandatory Y); 5 Window (days) / Window Starts From (Number, drop-down, mandatory Y); 6 Effective From / Effective To / Description (Date, text, mandatory Y / N / N).
+Fields in this order: 1 Insurer / Product Line / Segment / Rate / Window / Effective / Status (Column, mandatory -); 2 Insurer / Product Line / Segment (Drop-down, mandatory Y / N / N); 3 Product Line (blank = all) / Segment (blank = all) (Text, mandatory N); 4 Rate (% of basic premium) (Number, mandatory Y); 5 Window (days) / Window Starts From (Number, drop-down, mandatory Y); 6 Effective From / Effective To / Description (Date, text, mandatory Y / N / N).
 Actions: New Rule / Save Rule.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -37398,7 +37398,7 @@
         <is>
           <t>The screen matches SCR-OP-36 Disbursement Queue of the FRS.
 Fields in this order: 1 To Acknowledge / Acknowledged / DV Assigned / Paid / Returned / Cancelled (Tab, mandatory -); 2 Request No. / Payee / From / Amount / DV No. / Sent / Status (Column, mandatory -); 3 Disbursement Voucher No. (Text, mandatory Y); 4 Reason for Return (Text, mandatory Y).
-Actions: Acknowledge; Assign DV / Assign DV Number; Mark Paid; Return / Return Request.
+Actions: Acknowledge; Assign DV / Assign DV Number; Mark Paid; Return to Sender / Return Request.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -37634,7 +37634,7 @@
       <c r="L325" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-39 Endorsement Request of the FRS.
-Fields in this order: 1 Policy No. / ARN / Invoice (Reference chip, mandatory -); 2 Stage pill (Status pill, mandatory -); 3 Policy No. / Invoice / Insurer / Product / Period / Effective / Type / Requested By / Aging / Placement Slip / Batch (Display, mandatory -); 4 Endorsement workflow header (Stepper, mandatory -); 5 Details / Policy / Recompute / Accounting / Policy Transactions / Documents / History (Tab, mandatory -); 6 Endorsement Type / Request Type / Reason / Effective Date / Refund Basis / Sum Insured Change / Insurer Endorsement Ref. / New Period / Description / Instructions / Duplicate Justification / Baseline Justification / Quotation (Display, mandatory -); 7 Requested By / Submitted / Validated / Approved / Posted / Completed / Aging / Endorsement Slip (Display, mandatory -); 8 ARN / Placement Slip / Client / Insurer / Product / Period of Cover / Gross Premium (Display, mandatory -); 9 Before and After / Per Insurer (Table, mandatory -); 10 Journal / GL Account / Party / Debit / Credit (Column, mandatory -); 11 Date / Transaction / Reference / Premium Change / Taxes Change / Commission Change / Gross Premium After / Status / Accounting (Column, mandatory -); 12 Documents panel (Panel, mandatory -); 13 Quotation No. (Text, mandatory Y).
+Fields in this order: 1 Policy No. / ARN / Invoice (Reference chip, mandatory -); 2 Stage pill (Status pill, mandatory -); 3 Policy No. / Invoice / Insurer / Product / Period / Effective / Type / Requested By / Aging / Placement Slip / Batch (Display, mandatory -); 4 Endorsement workflow header (Stepper, mandatory -); 5 Details / Policy / Recompute / Accounting / Policy Transactions / Documents / History (Tab, mandatory -); 6 Endorsement Type / Request Type / Reason / Effective Date / Refund Basis / Sum Insured Change / Insurer Endorsement Ref. / New Period / Description / Instructions / Duplicate Justification / Baseline Justification / Quotation (Display, mandatory -); 7 Requested By / Submitted / Validated / Approved / Posted / Completed / Aging / Endorsement Slip (Display, mandatory -); 8 ARN / Placement Slip / Client / Insurer / Product / Period of Cover / Gross Premium (Display, mandatory -); 9 Before and After / Per Insurer (Table, mandatory -); 10 Journal / GL Account / Party / Debit / Credit (Column, mandatory -); 11 Date / Transaction / Reference / Premium Change / Taxes / Commission / Gross Premium After / Status / Accounting (Column, mandatory -); 12 Documents panel (Panel, mandatory -); 13 Quotation No. (Text, mandatory Y).
 Actions: Edit; Submit for Validation / Resubmit; Validate; Approve; Return to Requester; Post; Re-apply Payments; Link Quotation; Cancel request; Endorsement Slip / Validation Slip.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -38027,7 +38027,7 @@
       <c r="L330" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-44 Reconciliation Cycles of the FRS.
-Fields in this order: 1 All / Extracted / Sent to Insurer / Reconciling / Closed (Tab, mandatory -); 2 Search Insurer Code (Text, mandatory N); 3 Cycle No. / Insurer / Production Month / Items / BDOI Only / Insurer Only / Matched / Sent / Last Feedback / Stage (Column, mandatory -).
+Fields in this order: 1 All / Extracted / Sent to Insurer / Reconciling / Closed (Tab, mandatory -); 2 Insurer (Drop-down, mandatory N); 3 Cycle No. / Insurer / Production Month / Items / BDOI Only / Insurer Only / Matched / Sent / Last Feedback / Stage (Column, mandatory -).
 Actions: Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -38107,7 +38107,7 @@
         <is>
           <t>The screen matches SCR-OP-45 Reconciliation Cycle of the FRS.
 Fields in this order: 1 Cycle chip and stage pill (Reference chip, status pill, mandatory -); 2 Production Month / Items / Matched / BDOI Only / Insurer Only / Sent to Insurer / Last Feedback (Display, mandatory -); 3 Reconciliation workflow header (Stepper, mandatory -); 4 Items / Registers Sent / Early Incentive / Documents (Tab, mandatory -); 5 Bucket tabs (Tab, mandatory -); 6 Search Invoice, Policy or Assured (Text, mandatory N); 7 Marketing AO / AB / Sales Unit / Market Segment / Product Line (Filter, mandatory N); 8 Invoice / Policy / Assured / AO / Gross Premium (BDOI / Insurer) / Differences / Disposition / Status (Column, mandatory -); 9 Policy No. / Invoice / Reference No. / Assured Name / Period From / Period To / Basic Premium / Gross Premium / Commission (Display, mandatory -); 10 Company Concerned / Disposition / Instruction / Insurer Feedback / Marketing Feedback (Drop-down, text, mandatory N); 11 Company Concerned / Disposition (Drop-down, mandatory Y (disposition)); 12 Insurer Line (Drop-down, mandatory Y); 13 Extract No. / Trigger / Booking Period / Accounts / New / Extracted / Sent (Column, mandatory -); 14 Invoice No. / Assured / Inception / Remitted / Days / Expected / Per Insurer / Outcome (Column, mandatory -); 15 Comment (Text area, mandatory N).
-Actions: Run Matching; Save Feedback; Set Disposition / Apply to Selected; Pair / Pair Items; Split Pairing; Close Cycle.
+Actions: Run Matching; Save Feedback; Set Disposition / Apply to Selected; Pair with Another Item / Pair Items; Split Pairing; Close Cycle.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -38185,8 +38185,8 @@
       <c r="L332" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-46 Production Extracts of the FRS.
-Fields in this order: 1 Search Insurer Code (Text, mandatory N); 2 Extract No. / Trigger / Booking Period / Accounts / New / Extracted / Sent (Column, mandatory -); 3 Insurer Code / Production Month (Text, month, mandatory Y); 4 To / Cc (Text, mandatory Y / N).
-Actions: New Extract / Extract Register; Download; Send to Insurer / Resend.
+Fields in this order: 1 Insurer (Drop-down, mandatory N); 2 Extract No. / Trigger / Booking Period / Accounts / New / Extracted / Sent (Column, mandatory -); 3 Insurer / Production Month (Drop-down, month (MMM-yyyy), mandatory Y); 4 To / Cc (Text, mandatory Y / N).
+Actions: New Extract / Extract Register; Download; Send to Insurer / Resend to Insurer.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -38264,7 +38264,7 @@
       <c r="L333" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-47 Insurer Feedback of the FRS.
-Fields in this order: 1 Search Insurer Code (Text, mandatory N); 2 File / Insurer / Production Month / Rows Read / Accepted / Failed / Message / Uploaded / Status (Column, mandatory -); 3 Insurer Feedback File (File, mandatory Y).
+Fields in this order: 1 Insurer (Drop-down, mandatory N); 2 File / Insurer / Production Month / Rows Read / Accepted / Failed / Message / Uploaded / Status (Column, mandatory -); 3 Insurer Feedback File (File, mandatory Y).
 Actions: Upload Feedback / Upload and Match.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -38422,7 +38422,7 @@
       <c r="L335" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-49 Extract Schedules of the FRS.
-Fields in this order: 1 Insurer / Frequency / Next Run / Auto Send / Recipients / Last Run / Status (Column, mandatory -); 2 Insurer Code (Text, mandatory Y); 3 Frequency / Run Day (Drop-down, number, mandatory Y); 4 Recipients (Text, mandatory N); 5 Send automatically (Check box, mandatory N).
+Fields in this order: 1 Insurer / Frequency / Next Run / Auto Send / Recipients / Last Run / Status (Column, mandatory -); 2 Insurer (Drop-down, mandatory Y); 3 Frequency / Run Day (Drop-down, number, mandatory Y); 4 Recipients (Text, mandatory N); 5 Send automatically (Check box, mandatory N).
 Actions: New Schedule / Save Schedule.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -38736,7 +38736,7 @@
       <c r="L339" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-53 DP Billings of the FRS.
-Fields in this order: 1 To Send / Awaiting Insurer / To Collect / Returned to Collection / Closed / Cancelled (Tab, mandatory -); 2 Search Insurer Code (Text, mandatory N); 3 Billing No. / Insurer / Accounts / Net Commission / Sent / Answer Due / Handler / Stage (Column, mandatory -).
+Fields in this order: 1 To Send / Awaiting Insurer / To Collect / Returned to Collection / Closed / Cancelled (Tab, mandatory -); 2 Insurer (Drop-down, mandatory N); 3 Billing No. / Insurer / Accounts / Net Commission / Sent / Answer Due / Handler / Stage (Column, mandatory -).
 Actions: Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -38973,7 +38973,7 @@
       <c r="L342" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-56 Incentive Schemes of the FRS.
-Fields in this order: 1 Scheme / Type / Insurer / Period / Beneficiary / Tiers / Effective / Status (Column, mandatory -); 2 Code / Name (Text, mandatory Y); 3 Scheme Type (Drop-down, mandatory Y); 4 Calculation (Drop-down, mandatory Y); 5 Period / Beneficiary (Drop-down, mandatory Y); 6 Insurer Code / Segments / Product Lines (Text, mandatory N); 7 Effective From / Effective To (Date, mandatory Y / N); 8 Production Target / Rate % / Multiplier / Minimum Basic Premium / Amount per Policy (Number, mandatory Cond.: an active scheme needs one tier).
+Fields in this order: 1 Scheme / Type / Insurer / Period / Beneficiary / Tiers / Effective / Status (Column, mandatory -); 2 Name (Text, mandatory Y); 3 Scheme Type (Drop-down, mandatory Y); 4 Calculation (Drop-down, mandatory Y); 5 Period / Beneficiary (Drop-down, mandatory Y); 6 Insurer / Segments / Product Lines (Drop-down, text, mandatory N); 7 Effective From / Effective To (Date, mandatory Y / N); 8 Production Target / Rate % / Multiplier / Minimum Basic Premium / Amount per Policy (Number, mandatory Cond.: an active scheme needs one tier).
 Actions: New Scheme / Save Scheme; Add Tier / Remove.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -39131,7 +39131,7 @@
       <c r="L344" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-58 BIR Certificates of the FRS.
-Fields in this order: 1 Submitted / Rejected / Acknowledged (Tab, mandatory -); 2 Submission No. / Insurer / Period / Tax Withheld / ORs / Submitted / Status (Column, mandatory -); 3 Insurer Code / BIR Form / Certificate No. (Text, mandatory Y); 4 Tax Withheld / Period From / Period To (Number, date, mandatory Y); 5 Official receipts covered (Table, mandatory Y).
+Fields in this order: 1 Submitted / Rejected / Acknowledged (Tab, mandatory -); 2 Submission No. / Insurer / Period / Tax Withheld / ORs / Submitted / Status (Column, mandatory -); 3 Insurer / BIR Form / Certificate No. (Drop-down, text, mandatory Y); 4 Tax Withheld / Period From / Period To (Number, date, mandatory Y); 5 Official receipts covered (Table, mandatory Y).
 Actions: Submit Certificate / Submit to Comptrollership; Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -39368,7 +39368,7 @@
       <c r="L347" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-61 Interfaces of the FRS.
-Fields in this order: 1 Feeds / Run Log (Tab, mandatory -); 2 Feed / Partner / Transport / Owner / Schedule / Status (Column, mandatory -); 3 Run No. / Feed / Trigger / Started / Read / OK / Duplicate / Failed / File / Status (Column, mandatory -); 4 Record / Status / Created / Message / Received (Column, mandatory -); 5 [Schedule] / Active (Text, check box, mandatory N); 6 File (File, mandatory Y); 7 Invoice number or ARN (Text, mandatory N).
+Fields in this order: 1 Feeds / Run Log (Tab, mandatory -); 2 Feed / Partner / Transport / Owner / Schedule / Status (Column, mandatory -); 3 Run No. / Feed / Trigger / Started / Read / OK / Duplicate / Failed / File / Status (Column, mandatory -); 4 Record / Status / Created / Message / Received (Column, mandatory -); 5 Runs / Time / Active (Drop-down, time, check box, mandatory N); 6 File (File, mandatory Y); 7 Invoice number or ARN (Text, mandatory N).
 Actions: Configure / Save Feed; Upload File; Replay Booked Invoices / Replay Invoices; Open a run.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -39447,7 +39447,7 @@
       <c r="L348" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-OP-62 FFY Register of the FRS.
-Fields in this order: 1 ARN / Client / Product / Insurer (Column, mandatory -); 2 Period (Column, mandatory -); 3 Gross Premium / Status / Flags (Column, mandatory -); 4 FFY Start / FFY End (Column, mandatory -); 5 Officer (Column, mandatory -).
+Fields in this order: 1 ARN / Client / Product / Insurer (Column, mandatory -); 2 Period (Column, mandatory -); 3 Gross Premium / Status / Flags (Column, mandatory -); 4 FFY Period (Column, mandatory -); 5 Officer (Column, mandatory -).
 Actions: Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -40071,18 +40071,18 @@
       <c r="L356" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-054: "The requested action is applied to the receipt."
-MSG-OP-055: "The requester cannot approve &lt;transaction no&gt;" (MAKER_CHECKER_VIOLATION)
-MSG-OP-056: "&lt;transaction no&gt; is &lt;stage&gt;" (RECEIPT_ACTION_NOT_FOR_APPROVAL)
-MSG-OP-057: "Receipt &lt;receipt no&gt; already has a request waiting for approval" (RECEIPT_ACTION_PENDING)
-MSG-OP-058: "Receipt &lt;receipt no&gt; is already cancelled" (RECEIPT_ALREADY_CANCELLED)
-MSG-OP-059: "Unapplied item &lt;reference&gt; of the receipt is &lt;stage&gt;" (RECEIPT_HAS_DISPOSITION)
-MSG-OP-060: "Only a cancelled receipt can be reinstated" (RECEIPT_NOT_CANCELLED)
-MSG-OP-061: "Select a reason" (RECEIPT_REASON_REQUIRED)
-MSG-OP-062: "Specify the reason when 'Others' is selected" (RECEIPT_REASON_TEXT_REQUIRED)
-MSG-OP-063: "The reinstated amount must be above zero and at most &lt;amount&gt;" (REINSTATEMENT_AMOUNT)
-MSG-OP-064: "Enter the &lt;missing&gt;" (REINSTATEMENT_FIELDS_REQUIRED)
-MSG-OP-065: "Premium reinstatement reasons apply to ARs" (REINSTATEMENT_REASON_GROUP)</t>
+MSG-OP-052: "The requested action is applied to the receipt."
+MSG-OP-053: "The requester cannot approve &lt;transaction no&gt;" (MAKER_CHECKER_VIOLATION)
+MSG-OP-054: "&lt;transaction no&gt; is &lt;stage&gt;" (RECEIPT_ACTION_NOT_FOR_APPROVAL)
+MSG-OP-055: "Receipt &lt;receipt no&gt; already has a request waiting for approval" (RECEIPT_ACTION_PENDING)
+MSG-OP-056: "Receipt &lt;receipt no&gt; is already cancelled" (RECEIPT_ALREADY_CANCELLED)
+MSG-OP-057: "Unapplied item &lt;reference&gt; of the receipt is &lt;stage&gt;" (RECEIPT_HAS_DISPOSITION)
+MSG-OP-058: "Only a cancelled receipt can be reinstated" (RECEIPT_NOT_CANCELLED)
+MSG-OP-059: "Select a reason" (RECEIPT_REASON_REQUIRED)
+MSG-OP-060: "Specify the reason when 'Others' is selected" (RECEIPT_REASON_TEXT_REQUIRED)
+MSG-OP-061: "The reinstated amount must be above zero and at most &lt;amount&gt;" (REINSTATEMENT_AMOUNT)
+MSG-OP-062: "Enter the &lt;missing&gt;" (REINSTATEMENT_FIELDS_REQUIRED)
+MSG-OP-063: "Premium reinstatement reasons apply to ARs" (REINSTATEMENT_REASON_GROUP)</t>
         </is>
       </c>
       <c r="M356" s="12" t="inlineStr">
@@ -40157,21 +40157,21 @@
       <c r="L357" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-068: "The amount must be above zero and at most the balance &lt;balance&gt;" (DISPOSITION_AMOUNT)
-MSG-OP-069: "Invoice &lt;invoice no&gt; takes no client payment" (DISPOSITION_INVOICE_NOT_RECEIVABLE)
-MSG-OP-070: "Unknown invoice &lt;invoice no&gt;" (DISPOSITION_INVOICE_UNKNOWN)
-MSG-OP-071: "&lt;description&gt; needs the team leader's approval and is not processed at once" (DISPOSITION_NEEDS_APPROVAL)
-MSG-OP-072: "Invoice &lt;target invoice no&gt; has nothing outstanding to apply to" (DISPOSITION_NOTHING_TO_APPLY)
-MSG-OP-073: "No application" (DISPOSITION_NO_APPLICATION)
-MSG-OP-074: "Enter &lt;what&gt;" (DISPOSITION_TARGET_REQUIRED)
-MSG-OP-075: "Disposition type &lt;type code&gt; has no processing rule" (DISPOSITION_TYPE_NOT_CONFIGURED)
-MSG-OP-076: "A reclass or transfer moves the whole balance &lt;balance&gt;" (DISPOSITION_WHOLE_BALANCE)
-MSG-OP-077: "The requester cannot approve the disposition" (MAKER_CHECKER_VIOLATION)
-MSG-OP-078: "A refund is reversed only after Disbursement returned the request" (REFUND_NOT_RETURNED)
-MSG-OP-079: "Enter the reason for the reversal" (REVERSAL_REASON_REQUIRED)
-MSG-OP-080: "An unapplied item needs an amount above zero" (UNAPPLIED_AMOUNT)
-MSG-OP-081: "Amount &lt;value&gt; is above the unapplied balance &lt;balance&gt; of &lt;reference&gt;" (UNAPPLIED_BALANCE_EXCEEDED)
-MSG-OP-082: "&lt;reference&gt; is &lt;stage&gt;, not &lt;stage&gt;" (UNAPPLIED_WRONG_STAGE)</t>
+MSG-OP-066: "The amount must be above zero and at most the balance &lt;balance&gt;" (DISPOSITION_AMOUNT)
+MSG-OP-067: "Invoice &lt;invoice no&gt; takes no client payment" (DISPOSITION_INVOICE_NOT_RECEIVABLE)
+MSG-OP-068: "Unknown invoice &lt;invoice no&gt;" (DISPOSITION_INVOICE_UNKNOWN)
+MSG-OP-069: "&lt;description&gt; needs the team leader's approval and is not processed at once" (DISPOSITION_NEEDS_APPROVAL)
+MSG-OP-070: "Invoice &lt;target invoice no&gt; has nothing outstanding to apply to" (DISPOSITION_NOTHING_TO_APPLY)
+MSG-OP-071: "No application" (DISPOSITION_NO_APPLICATION)
+MSG-OP-072: "Enter &lt;what&gt;" (DISPOSITION_TARGET_REQUIRED)
+MSG-OP-073: "Disposition type &lt;type code&gt; has no processing rule" (DISPOSITION_TYPE_NOT_CONFIGURED)
+MSG-OP-074: "A reclass or transfer moves the whole balance &lt;balance&gt;" (DISPOSITION_WHOLE_BALANCE)
+MSG-OP-075: "The requester cannot approve the disposition" (MAKER_CHECKER_VIOLATION)
+MSG-OP-076: "A refund is reversed only after Disbursement returned the request" (REFUND_NOT_RETURNED)
+MSG-OP-077: "Enter the reason for the reversal" (REVERSAL_REASON_REQUIRED)
+MSG-OP-078: "An unapplied item needs an amount above zero" (UNAPPLIED_AMOUNT)
+MSG-OP-079: "Amount &lt;value&gt; is above the unapplied balance &lt;balance&gt; of &lt;reference&gt;" (UNAPPLIED_BALANCE_EXCEEDED)
+MSG-OP-080: "&lt;reference&gt; is &lt;stage&gt;, not &lt;stage&gt;" (UNAPPLIED_WRONG_STAGE)</t>
         </is>
       </c>
       <c r="M357" s="12" t="inlineStr">
@@ -40246,20 +40246,20 @@
       <c r="L358" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-083: "Enter an amount above zero and at most the unapplied balance"
-MSG-OP-084: "Enter the client to reclass to"
-MSG-OP-085: "Enter the marketing unit to transfer to"
-MSG-OP-089: "The selected receipt is reversed as requested."
-MSG-OP-090: "&lt;request no&gt; is already &lt;status&gt;" (COLLECTOR_REQUEST_DECIDED)
-MSG-OP-091: "Disposition type &lt;type&gt; does not carry out a &lt;action&gt; request" (COLLECTOR_REQUEST_TYPE_MISMATCH)
-MSG-OP-092: "Unknown disposition type &lt;type&gt;" (DISPOSITION_TYPE_NOT_CONFIGURED)
-MSG-OP-093: "The requester cannot approve the payment reversal" (MAKER_CHECKER_VIOLATION)
-MSG-OP-094: "&lt;request no&gt; is already &lt;status&gt;" (PAYMENT_REVERSAL_DECIDED)
-MSG-OP-095: "Receipt &lt;receipt no&gt; has &lt;available&gt; applied to &lt;invoice no&gt;, less than &lt;target&gt;" (PAYMENT_REVERSAL_NOTHING_APPLIED)
-MSG-OP-096: "Unknown receipt &lt;receipt no&gt;" (PAYMENT_REVERSAL_RECEIPT_UNKNOWN)
-MSG-OP-097: "&lt;task no&gt; is already &lt;status&gt;" (REFUND_VALIDATION_DONE)
-MSG-OP-098: "Choose the unapplied item that holds the returned premium" (REFUND_VALIDATION_ITEM_REQUIRED)
-MSG-OP-099: "Enter the reason for rejecting" (REJECT_REASON_REQUIRED)</t>
+MSG-OP-081: "Enter an amount above zero and at most the unapplied balance"
+MSG-OP-082: "Enter the client to reclass to"
+MSG-OP-083: "Enter the marketing unit to transfer to"
+MSG-OP-087: "The selected receipt is reversed as requested."
+MSG-OP-088: "&lt;request no&gt; is already &lt;status&gt;" (COLLECTOR_REQUEST_DECIDED)
+MSG-OP-089: "Disposition type &lt;type&gt; does not carry out a &lt;action&gt; request" (COLLECTOR_REQUEST_TYPE_MISMATCH)
+MSG-OP-090: "Unknown disposition type &lt;type&gt;" (DISPOSITION_TYPE_NOT_CONFIGURED)
+MSG-OP-091: "The requester cannot approve the payment reversal" (MAKER_CHECKER_VIOLATION)
+MSG-OP-092: "&lt;request no&gt; is already &lt;status&gt;" (PAYMENT_REVERSAL_DECIDED)
+MSG-OP-093: "Receipt &lt;receipt no&gt; has &lt;available&gt; applied to &lt;invoice no&gt;, less than &lt;target&gt;" (PAYMENT_REVERSAL_NOTHING_APPLIED)
+MSG-OP-094: "Unknown receipt &lt;receipt no&gt;" (PAYMENT_REVERSAL_RECEIPT_UNKNOWN)
+MSG-OP-095: "&lt;task no&gt; is already &lt;status&gt;" (REFUND_VALIDATION_DONE)
+MSG-OP-096: "Choose the unapplied item that holds the returned premium" (REFUND_VALIDATION_ITEM_REQUIRED)
+MSG-OP-097: "Enter the reason for rejecting" (REJECT_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M358" s="12" t="inlineStr">
@@ -40334,7 +40334,7 @@
       <c r="L359" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-101: "Pre-booked payment of &lt;arn&gt; is &lt;status&gt;" (PREBOOKED_NOT_OPEN)</t>
+MSG-OP-099: "Pre-booked payment of &lt;arn&gt; is &lt;status&gt;" (PREBOOKED_NOT_OPEN)</t>
         </is>
       </c>
       <c r="M359" s="12" t="inlineStr">
@@ -40409,11 +40409,11 @@
       <c r="L360" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-105: "A delimited layout needs a one-character separator" (PAYMENT_LAYOUT_DELIMITER)
-MSG-OP-106: "A fixed-width layout needs its fields" (PAYMENT_LAYOUT_FIELDS)
-MSG-OP-107: "Start and length of '&lt;part&gt;' must be numbers" (PAYMENT_LAYOUT_FIELDS)
-MSG-OP-108: "Write each field as Header:start:length, not '&lt;part&gt;'" (PAYMENT_LAYOUT_FIELDS)
-MSG-OP-109: "Unknown layout kind &lt;new kind&gt;" (PAYMENT_LAYOUT_KIND)</t>
+MSG-OP-103: "A delimited layout needs a one-character separator" (PAYMENT_LAYOUT_DELIMITER)
+MSG-OP-104: "A fixed-width layout needs its fields" (PAYMENT_LAYOUT_FIELDS)
+MSG-OP-105: "Start and length of '&lt;part&gt;' must be numbers" (PAYMENT_LAYOUT_FIELDS)
+MSG-OP-106: "Write each field as Header:start:length, not '&lt;part&gt;'" (PAYMENT_LAYOUT_FIELDS)
+MSG-OP-107: "Unknown layout kind &lt;new kind&gt;" (PAYMENT_LAYOUT_KIND)</t>
         </is>
       </c>
       <c r="M360" s="12" t="inlineStr">
@@ -40488,11 +40488,11 @@
       <c r="L361" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-110: "Enter an amount above zero"
-MSG-OP-112: "A post-dated check needs an amount above zero" (PDC_AMOUNT)
-MSG-OP-113: "Check &lt;bank code&gt; &lt;check no&gt; is already warehoused" (PDC_DUPLICATE)
-MSG-OP-114: "Check &lt;warehouse no&gt; is &lt;status&gt;, not in the warehouse" (PDC_NOT_WAREHOUSED)
-MSG-OP-115: "A check leaves the warehouse as returned, replaced or pulled out" (PDC_RELEASE_STATUS)</t>
+MSG-OP-108: "Enter an amount above zero"
+MSG-OP-110: "A post-dated check needs an amount above zero" (PDC_AMOUNT)
+MSG-OP-111: "Check &lt;bank code&gt; &lt;check no&gt; is already warehoused" (PDC_DUPLICATE)
+MSG-OP-112: "Check &lt;warehouse no&gt; is &lt;status&gt;, not in the warehouse" (PDC_NOT_WAREHOUSED)
+MSG-OP-113: "A check leaves the warehouse as returned, replaced or pulled out" (PDC_RELEASE_STATUS)</t>
         </is>
       </c>
       <c r="M361" s="12" t="inlineStr">
@@ -40567,13 +40567,13 @@
       <c r="L362" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-117: "The pickup is cancelled and the check stays with the cashier."
-MSG-OP-118: "The check amount must be above zero" (PICKUP_AMOUNT)
-MSG-OP-119: "Unknown company &lt;"company"&gt;" (PICKUP_COMPANY_UNKNOWN)
-MSG-OP-120: "Collection reference &lt;collection ref&gt; is already queued" (PICKUP_DUPLICATE)
-MSG-OP-121: "None of the selected requests is due for printing" (PICKUP_NOTHING_DUE)
-MSG-OP-122: "Pick-up request &lt;collection ref&gt; is &lt;status&gt;" (PICKUP_NOT_QUEUED)
-MSG-OP-123: "Pick-up record &lt;key&gt; is incomplete: &lt;message&gt;" (PICKUP_RECORD_INVALID)</t>
+MSG-OP-115: "The pick-up is cancelled and the check stays with the client."
+MSG-OP-116: "The check amount must be above zero" (PICKUP_AMOUNT)
+MSG-OP-117: "Unknown company &lt;"company"&gt;" (PICKUP_COMPANY_UNKNOWN)
+MSG-OP-118: "Collection reference &lt;collection ref&gt; is already queued" (PICKUP_DUPLICATE)
+MSG-OP-119: "None of the selected requests is due for printing" (PICKUP_NOTHING_DUE)
+MSG-OP-120: "Pick-up request &lt;collection ref&gt; is &lt;status&gt;" (PICKUP_NOT_QUEUED)
+MSG-OP-121: "Pick-up record &lt;key&gt; is incomplete: &lt;message&gt;" (PICKUP_RECORD_INVALID)</t>
         </is>
       </c>
       <c r="M362" s="12" t="inlineStr">
@@ -40648,9 +40648,9 @@
       <c r="L363" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-127: "Receipt &lt;receipt no&gt; is cancelled" (COP_CANCELLED_RECEIPT)
-MSG-OP-128: "&lt;batch no&gt; has no failures" (PRINT_NOTHING_FAILED)
-MSG-OP-129: "Select between 1 and 500 receipts to print" (PRINT_SELECTION)</t>
+MSG-OP-125: "Receipt &lt;receipt no&gt; is cancelled" (COP_CANCELLED_RECEIPT)
+MSG-OP-126: "&lt;batch no&gt; has no failures" (PRINT_NOTHING_FAILED)
+MSG-OP-127: "Select between 1 and 500 receipts to print" (PRINT_SELECTION)</t>
         </is>
       </c>
       <c r="M363" s="12" t="inlineStr">
@@ -40725,22 +40725,22 @@
       <c r="L364" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-132: "Certificate number is required for a certificate"
-MSG-OP-133: "Enter an amount above zero, or leave it empty for the expected 2%"
-MSG-OP-134: "Invoice number is required"
-MSG-OP-137: "The selected certificates are validated and the 2307 report is posted."
-MSG-OP-138: "Invoice &lt;invoice no&gt; already has a 2307 tag in process" (CWT_ALREADY_TAGGED)
-MSG-OP-139: "Invoice &lt;invoice no&gt; has no 2% CWT portion outstanding" (CWT_AMOUNT)
-MSG-OP-140: "&lt;ref&gt;: the invoice has less premium outstanding than the 2307 amount" (CWT_AMOUNT_MISMATCH)
-MSG-OP-141: "Select the 2307 tags to validate" (CWT_BATCH_EMPTY)
-MSG-OP-142: "A 2307 batch holds the certificates of one insurer" (CWT_BATCH_ONE_INSURER)
-MSG-OP-143: "&lt;batch no&gt; is &lt;status&gt;" (CWT_BATCH_ROUTED)
-MSG-OP-144: "&lt;reference&gt; is settled in cash" (CWT_CASH_IN_BATCH)
-MSG-OP-145: "A certificate tag needs the BIR 2307 certificate number" (CWT_CERTIFICATE_REQUIRED)
-MSG-OP-146: "The CWT copy of &lt;reference&gt; was not received" (CWT_COPY_MISSING)
-MSG-OP-147: "Unknown invoice &lt;invoice no&gt;" (CWT_INVOICE_UNKNOWN)
-MSG-OP-148: "&lt;reference&gt; is a certificate tag" (CWT_NOT_CASH)
-MSG-OP-149: "&lt;reference&gt; is &lt;stage&gt;" (CWT_WRONG_STAGE)</t>
+MSG-OP-130: "Certificate number is required for a certificate"
+MSG-OP-131: "Enter an amount above zero, or leave it empty for the expected 2%"
+MSG-OP-132: "Invoice number is required"
+MSG-OP-135: "The selected certificates are validated and the 2307 report is posted."
+MSG-OP-136: "Invoice &lt;invoice no&gt; already has a 2307 tag in process" (CWT_ALREADY_TAGGED)
+MSG-OP-137: "Invoice &lt;invoice no&gt; has no 2% CWT portion outstanding" (CWT_AMOUNT)
+MSG-OP-138: "&lt;ref&gt;: the invoice has less premium outstanding than the 2307 amount" (CWT_AMOUNT_MISMATCH)
+MSG-OP-139: "Select the 2307 tags to validate" (CWT_BATCH_EMPTY)
+MSG-OP-140: "A 2307 batch holds the certificates of one insurer" (CWT_BATCH_ONE_INSURER)
+MSG-OP-141: "&lt;batch no&gt; is &lt;status&gt;" (CWT_BATCH_ROUTED)
+MSG-OP-142: "&lt;reference&gt; is settled in cash" (CWT_CASH_IN_BATCH)
+MSG-OP-143: "A certificate tag needs the BIR 2307 certificate number" (CWT_CERTIFICATE_REQUIRED)
+MSG-OP-144: "The CWT copy of &lt;reference&gt; was not received" (CWT_COPY_MISSING)
+MSG-OP-145: "Unknown invoice &lt;invoice no&gt;" (CWT_INVOICE_UNKNOWN)
+MSG-OP-146: "&lt;reference&gt; is a certificate tag" (CWT_NOT_CASH)
+MSG-OP-147: "&lt;reference&gt; is &lt;stage&gt;" (CWT_WRONG_STAGE)</t>
         </is>
       </c>
       <c r="M364" s="12" t="inlineStr">
@@ -40815,7 +40815,7 @@
       <c r="L365" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-151: "Unknown company &lt;company&gt;" (FLOW_IN_COMPANY_UNKNOWN)</t>
+MSG-OP-149: "Unknown company &lt;company&gt;" (FLOW_IN_COMPANY_UNKNOWN)</t>
         </is>
       </c>
       <c r="M365" s="12" t="inlineStr">
@@ -40890,10 +40890,10 @@
       <c r="L366" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-152: "&lt;run no&gt; failed: &lt;message&gt;"
-MSG-OP-154: "Invoice &lt;invoice no&gt; is not an invoice of &lt;insurer code&gt;" (REMIT_INVOICE_INSURER)
-MSG-OP-155: "Invoice &lt;invoice no&gt; cannot be extracted: remittance status &lt;remittance status&gt; (direct payment) / " (REMIT_INVOICE_NOT_EXTRACTABLE)
-MSG-OP-156: "Invoice &lt;invoice no&gt; cannot be remitted now: &lt;invoice no&gt;" (SPECIAL_REMIT_NOT_ELIGIBLE)</t>
+MSG-OP-150: "&lt;run no&gt; failed: &lt;message&gt;"
+MSG-OP-152: "Invoice &lt;invoice no&gt; is not an invoice of &lt;insurer code&gt;" (REMIT_INVOICE_INSURER)
+MSG-OP-153: "Invoice &lt;invoice no&gt; cannot be extracted: remittance status &lt;remittance status&gt; (direct payment) / " (REMIT_INVOICE_NOT_EXTRACTABLE)
+MSG-OP-154: "Invoice &lt;invoice no&gt; cannot be remitted now: &lt;invoice no&gt;" (SPECIAL_REMIT_NOT_ELIGIBLE)</t>
         </is>
       </c>
       <c r="M366" s="12" t="inlineStr">
@@ -40968,20 +40968,21 @@
       <c r="L367" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-158: "Hold Until is required"
-MSG-OP-159: "Hold Until must be a future date"
-MSG-OP-160: "Invoice No. is required"
-MSG-OP-163: "Select a reason"
-MSG-OP-164: "Batch &lt;batch no&gt; has no invoice left to remit" (REMIT_BATCH_EMPTY)
-MSG-OP-165: "Batch &lt;batch no&gt; can no longer return" (REMIT_BATCH_STAGE)
-MSG-OP-166: "Batch &lt;batch no&gt; is &lt;stage&gt;: lines can no longer change" (REMIT_BATCH_STAGE)
-MSG-OP-167: "Batch &lt;batch no&gt; must be approved by another user" (REMIT_FOUR_EYES)
-MSG-OP-168: "Invoice &lt;invoice no&gt; is already excluded" (REMIT_LINE_ALREADY_EXCLUDED)
-MSG-OP-169: "Invoice &lt;invoice no&gt; is not excluded" (REMIT_LINE_NOT_EXCLUDED)
-MSG-OP-170: "Invoice &lt;invoice no&gt; can no longer be restored (remittance status &lt;remittance status&gt; / , locked by &lt;lock owner&gt;)" (REMIT_RESTORE_NOT_ELIGIBLE)
-MSG-OP-171: "The schedule of &lt;batch no&gt; was already sent" (REMIT_SCHEDULE_ALREADY_SENT)
-MSG-OP-172: "The schedule of &lt;batch no&gt; can be sent once the batch is approved" (REMIT_SCHEDULE_NOT_APPROVED)
-MSG-OP-173: "Batch &lt;batch no&gt; cannot go on: &lt;problems&gt;" (REMIT_SUBMISSION_INVALID)</t>
+MSG-OP-156: "Check within the holding period"
+MSG-OP-157: "Hold Until is required"
+MSG-OP-158: "Hold Until must be a future date"
+MSG-OP-159: "Invoice No. is required"
+MSG-OP-162: "Select a reason"
+MSG-OP-163: "Batch &lt;batch no&gt; has no invoice left to remit" (REMIT_BATCH_EMPTY)
+MSG-OP-164: "Batch &lt;batch no&gt; can no longer return" (REMIT_BATCH_STAGE)
+MSG-OP-165: "Batch &lt;batch no&gt; is &lt;stage&gt;: lines can no longer change" (REMIT_BATCH_STAGE)
+MSG-OP-166: "Batch &lt;batch no&gt; must be approved by another user" (REMIT_FOUR_EYES)
+MSG-OP-167: "Invoice &lt;invoice no&gt; is already excluded" (REMIT_LINE_ALREADY_EXCLUDED)
+MSG-OP-168: "Invoice &lt;invoice no&gt; is not excluded" (REMIT_LINE_NOT_EXCLUDED)
+MSG-OP-169: "Invoice &lt;invoice no&gt; can no longer be restored (remittance status &lt;remittance status&gt; / , locked by &lt;lock owner&gt;)" (REMIT_RESTORE_NOT_ELIGIBLE)
+MSG-OP-170: "The schedule of &lt;batch no&gt; was already sent" (REMIT_SCHEDULE_ALREADY_SENT)
+MSG-OP-171: "The schedule of &lt;batch no&gt; can be sent once the batch is approved" (REMIT_SCHEDULE_NOT_APPROVED)
+MSG-OP-172: "Batch &lt;batch no&gt; cannot go on: &lt;problems&gt;" (REMIT_SUBMISSION_INVALID)</t>
         </is>
       </c>
       <c r="M367" s="12" t="inlineStr">
@@ -41056,14 +41057,14 @@
       <c r="L368" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-175: "The file must have the columns &lt;required&gt;" (FEED_FILE_COLUMNS)
-MSG-OP-176: "The file has no lines" (FEED_FILE_EMPTY)
-MSG-OP-177: "Line &lt;line no&gt;: &lt;column&gt; must be YYYY-MM-DD" (FEED_VALUE_INVALID)
-MSG-OP-178: "Line &lt;line no&gt;: &lt;column&gt; must be an amount" (FEED_VALUE_INVALID)
-MSG-OP-179: "Line &lt;line no&gt;: &lt;column&gt; is missing" (FEED_VALUE_MISSING)
-MSG-OP-180: "Batch &lt;batch no&gt; is &lt;stage&gt;: not yet approved" (REMIT_OR_BATCH_STAGE)
-MSG-OP-181: "OR &lt;number&gt; was already recorded for client &lt;client code&gt;" (REMIT_OR_DUPLICATE)
-MSG-OP-182: "Invoice &lt;invoice no&gt; was excluded from &lt;batch no&gt;" (REMIT_OR_LINE_EXCLUDED)</t>
+MSG-OP-174: "The file must have the columns &lt;details&gt;" (FEED_FILE_COLUMNS)
+MSG-OP-175: "The file has no lines" (FEED_FILE_EMPTY)
+MSG-OP-176: "Line &lt;line no&gt;: &lt;column&gt; must be a date such as 28-Oct-2026" (FEED_VALUE_INVALID)
+MSG-OP-177: "Line &lt;line no&gt;: &lt;column&gt; must be an amount" (FEED_VALUE_INVALID)
+MSG-OP-178: "Line &lt;line no&gt;: &lt;column&gt; is missing" (FEED_VALUE_MISSING)
+MSG-OP-179: "Batch &lt;batch no&gt; is &lt;stage&gt;: not yet approved" (REMIT_OR_BATCH_STAGE)
+MSG-OP-180: "OR &lt;number&gt; was already recorded for client &lt;client code&gt;" (REMIT_OR_DUPLICATE)
+MSG-OP-181: "Invoice &lt;invoice no&gt; was excluded from &lt;batch no&gt;" (REMIT_OR_LINE_EXCLUDED)</t>
         </is>
       </c>
       <c r="M368" s="12" t="inlineStr">
@@ -41138,15 +41139,15 @@
       <c r="L369" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-184: "&lt;processor&gt; is not an active remittance processor" (HOLD_ASSIGNEE_NOT_ELIGIBLE)
-MSG-OP-185: "The hold-until date must be in the future" (HOLD_DATE)
-MSG-OP-186: "Invoice &lt;invoice no&gt; already has hold &lt;request no&gt;" (HOLD_DUPLICATE)
-MSG-OP-187: "The extension must be later than &lt;hold until&gt;" (HOLD_EXTENSION_DATE)
-MSG-OP-188: "Hold &lt;request no&gt; must be approved by another user" (HOLD_FOUR_EYES)
-MSG-OP-189: "Hold &lt;request no&gt; must be decided by another user" (HOLD_FOUR_EYES)
-MSG-OP-190: "Invoice &lt;invoice no&gt; cannot be held: remittance status &lt;remittance status&gt;" (HOLD_INVOICE_NOT_HOLDABLE)
-MSG-OP-191: "Hold &lt;request no&gt; is &lt;stage&gt;, not &lt;stage&gt;" (HOLD_STAGE)
-MSG-OP-192: "Hold &lt;request no&gt; is not active" (HOLD_STAGE)</t>
+MSG-OP-183: "&lt;processor&gt; is not an active remittance processor" (HOLD_ASSIGNEE_NOT_ELIGIBLE)
+MSG-OP-184: "The hold-until date must be in the future" (HOLD_DATE)
+MSG-OP-185: "Invoice &lt;invoice no&gt; already has hold &lt;request no&gt;" (HOLD_DUPLICATE)
+MSG-OP-186: "The extension must be later than &lt;hold until&gt;" (HOLD_EXTENSION_DATE)
+MSG-OP-187: "Hold &lt;request no&gt; must be approved by another user" (HOLD_FOUR_EYES)
+MSG-OP-188: "Hold &lt;request no&gt; must be decided by another user" (HOLD_FOUR_EYES)
+MSG-OP-189: "Invoice &lt;invoice no&gt; cannot be held: remittance status &lt;remittance status&gt;" (HOLD_INVOICE_NOT_HOLDABLE)
+MSG-OP-190: "Hold &lt;request no&gt; is &lt;stage&gt;, not &lt;stage&gt;" (HOLD_STAGE)
+MSG-OP-191: "Hold &lt;request no&gt; is not active" (HOLD_STAGE)</t>
         </is>
       </c>
       <c r="M369" s="12" t="inlineStr">
@@ -41221,9 +41222,9 @@
       <c r="L370" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-194: "Invoice &lt;invoice no&gt; already has request &lt;request no&gt;" (SPECIAL_REMIT_DUPLICATE)
-MSG-OP-195: "Request &lt;request no&gt; must be approved by another user" (SPECIAL_REMIT_FOUR_EYES)
-MSG-OP-196: "Invoice &lt;invoice no&gt; cannot be remitted specially: &lt;why&gt;" (SPECIAL_REMIT_NOT_ELIGIBLE)</t>
+MSG-OP-193: "Invoice &lt;invoice no&gt; already has request &lt;request no&gt;" (SPECIAL_REMIT_DUPLICATE)
+MSG-OP-194: "Request &lt;request no&gt; must be approved by another user" (SPECIAL_REMIT_FOUR_EYES)
+MSG-OP-195: "Invoice &lt;invoice no&gt; cannot be remitted specially: &lt;why&gt;" (SPECIAL_REMIT_NOT_ELIGIBLE)</t>
         </is>
       </c>
       <c r="M370" s="12" t="inlineStr">
@@ -41298,17 +41299,17 @@
       <c r="L371" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-199: "Choose the currency"
-MSG-OP-200: "Choose what the deduction settles"
-MSG-OP-201: "Enter a positive amount with at most 2 decimals"
-MSG-OP-202: "Insurer code is required"
-MSG-OP-205: "Source reference is required"
-MSG-OP-206: "The confirmation date cannot be in the future"
-MSG-OP-207: "Select the company" (COMPANY_REQUIRED)
-MSG-OP-208: "A deduction needs a positive amount" (REMIT_DEDUCTION_AMOUNT)
-MSG-OP-209: "Deduction &lt;deduction no&gt; must be confirmed by another user" (REMIT_DEDUCTION_FOUR_EYES)
-MSG-OP-210: "Deduction &lt;deduction no&gt; can only change as a draft" (REMIT_DEDUCTION_STAGE)
-MSG-OP-211: "Deduction &lt;deduction no&gt; needs the insurer's confirmation reference and date before submission" (REMIT_DEDUCTION_UNCONFIRMED)</t>
+MSG-OP-198: "Choose the currency"
+MSG-OP-199: "Choose what the deduction settles"
+MSG-OP-200: "Enter a positive amount with at most 2 decimals"
+MSG-OP-203: "Select the insurer"
+MSG-OP-204: "Source reference is required"
+MSG-OP-205: "The confirmation date cannot be in the future"
+MSG-OP-206: "Select the company" (COMPANY_REQUIRED)
+MSG-OP-207: "A deduction needs a positive amount" (REMIT_DEDUCTION_AMOUNT)
+MSG-OP-208: "Deduction &lt;deduction no&gt; must be confirmed by another user" (REMIT_DEDUCTION_FOUR_EYES)
+MSG-OP-209: "Deduction &lt;deduction no&gt; can only change as a draft" (REMIT_DEDUCTION_STAGE)
+MSG-OP-210: "Deduction &lt;deduction no&gt; needs the insurer's confirmation reference and date before submission" (REMIT_DEDUCTION_UNCONFIRMED)</t>
         </is>
       </c>
       <c r="M371" s="12" t="inlineStr">
@@ -41383,12 +41384,12 @@
       <c r="L372" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-213: "Insurer code is required"
-MSG-OP-214: "Rate must be above 0 and at most 100"
-MSG-OP-215: "The rule cannot end before it starts"
-MSG-OP-216: "Window must be 1 to 366 days"
-MSG-OP-217: "Choose the company of the rule" (COMPANY_REQUIRED)
-MSG-OP-218: "The rule cannot end before it starts" (INCENTIVE_RULE_PERIOD)</t>
+MSG-OP-212: "Rate must be above 0 and at most 100"
+MSG-OP-213: "Select the insurer"
+MSG-OP-214: "The rule cannot end before it starts"
+MSG-OP-215: "Window must be 1 to 366 days"
+MSG-OP-216: "Choose the company of the rule" (COMPANY_REQUIRED)
+MSG-OP-217: "The rule cannot end before it starts" (INCENTIVE_RULE_PERIOD)</t>
         </is>
       </c>
       <c r="M372" s="12" t="inlineStr">
@@ -41463,9 +41464,9 @@
       <c r="L373" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-221: "A payment request needs a positive amount" (DISBURSEMENT_AMOUNT)
-MSG-OP-222: "Too many references on one payment request" (DISBURSEMENT_REFERENCES)
-MSG-OP-223: "Payment request &lt;request no&gt; is &lt;status&gt; and cannot be &lt;action&gt;" (DISBURSEMENT_STATUS)</t>
+MSG-OP-219: "A payment request needs a positive amount" (DISBURSEMENT_AMOUNT)
+MSG-OP-220: "Too many references on one payment request" (DISBURSEMENT_REFERENCES)
+MSG-OP-221: "Payment request &lt;request no&gt; is &lt;status&gt; and cannot be &lt;action&gt;" (DISBURSEMENT_STATUS)</t>
         </is>
       </c>
       <c r="M373" s="12" t="inlineStr">
@@ -41540,31 +41541,31 @@
       <c r="L374" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-225: "A financial endorsement needs its request type"
-MSG-OP-227: "Describe the change"
-MSG-OP-228: "Enter at least one premium, charge or commission change"
-MSG-OP-229: "Enter the effective date"
-MSG-OP-230: "Enter the increase (positive) or decrease (negative)"
-MSG-OP-232: "Select the endorsement type"
-MSG-OP-233: "Select the reason for cancellation"
-MSG-OP-234: "The new expiry must be after the new inception"
-MSG-OP-235: "Enter the premium, charges or commission change" (ADJ_AMOUNTS_REQUIRED)
-MSG-OP-236: "Select the reason for cancellation" (ADJ_CANCELLATION_REASON_REQUIRED)
-MSG-OP-237: "Possible duplicate of &lt;details&gt; (same invoice, request type, reason and endorsement reference): give the justification to proceed" (ADJ_DUPLICATE_REQUEST)
-MSG-OP-238: "The effective date must be within the cover &lt;inception&gt; to &lt;expiry&gt;" (ADJ_EFFECTIVE_DATE_OUTSIDE_TERM)
-MSG-OP-239: "Request &lt;request no&gt; (&lt;computation&gt;) is still open on &lt;invoice no&gt;: a cancellation cannot be combined with another financial change" (ADJ_INCOMPATIBLE_REQUEST)
-MSG-OP-240: "Select at least one invoice" (ADJ_INVOICES_REQUIRED)
-MSG-OP-241: "Select between 1 and 50 invoices" (ADJ_INVOICES_REQUIRED)
-MSG-OP-242: "&lt;invoice no&gt; is cancelled or written off" (ADJ_INVOICE_CLOSED)
-MSG-OP-243: "A non-financial endorsement carries no request type, sum insured or amount change" (ADJ_NON_FINANCIAL_WITH_AMOUNTS)
-MSG-OP-244: "Enter a valid new period (a change of period keeps the term of &lt;inception&gt; to &lt;expiry&gt;)" (ADJ_PERIOD_INVALID)
-MSG-OP-245: "&lt;request no&gt; needs no quotation link" (ADJ_QUOTATION_NOT_REQUIRED)
-MSG-OP-246: "Enter the quotation number" (ADJ_QUOTATION_REF_REQUIRED)
-MSG-OP-247: "Enter the endorsement type, effective date and description" (ADJ_REQUEST_INCOMPLETE)
-MSG-OP-248: "Select the request type of a financial endorsement" (ADJ_REQUEST_TYPE_REQUIRED)
-MSG-OP-249: "&lt;invoice no&gt; is a return invoice: raise the request on the original" (ADJ_RETURN_INVOICE)
-MSG-OP-250: "Enter the increase or decrease of the total sum insured" (ADJ_TSI_CHANGE_REQUIRED)
-MSG-OP-251: "Endorsement type &lt;code&gt; has no class (FINANCIAL / NON_FINANCIAL)" (ADJ_TYPE_WITHOUT_CLASS)</t>
+MSG-OP-223: "A financial endorsement needs its request type"
+MSG-OP-225: "Describe the change"
+MSG-OP-226: "Enter at least one premium, charge or commission change"
+MSG-OP-227: "Enter the effective date"
+MSG-OP-228: "Enter the increase (positive) or decrease (negative)"
+MSG-OP-230: "Select the endorsement type"
+MSG-OP-231: "Select the reason for cancellation"
+MSG-OP-232: "The new expiry must be after the new inception"
+MSG-OP-233: "Enter the premium, charges or commission change" (ADJ_AMOUNTS_REQUIRED)
+MSG-OP-234: "Select the reason for cancellation" (ADJ_CANCELLATION_REASON_REQUIRED)
+MSG-OP-235: "Possible duplicate of &lt;details&gt; (same invoice, request type, reason and endorsement reference): give the justification to proceed" (ADJ_DUPLICATE_REQUEST)
+MSG-OP-236: "The effective date must be within the cover &lt;inception&gt; to &lt;expiry&gt;" (ADJ_EFFECTIVE_DATE_OUTSIDE_TERM)
+MSG-OP-237: "Request &lt;request no&gt; (&lt;&gt;) is still open on &lt;invoice no&gt;: a cancellation cannot be combined with another financial change" (ADJ_INCOMPATIBLE_REQUEST)
+MSG-OP-238: "Select at least one invoice" (ADJ_INVOICES_REQUIRED)
+MSG-OP-239: "Select between 1 and 50 invoices" (ADJ_INVOICES_REQUIRED)
+MSG-OP-240: "&lt;invoice no&gt; is cancelled or written off" (ADJ_INVOICE_CLOSED)
+MSG-OP-241: "A non-financial endorsement carries no request type, sum insured or amount change" (ADJ_NON_FINANCIAL_WITH_AMOUNTS)
+MSG-OP-242: "Enter a valid new period (a change of period keeps the term of &lt;inception&gt; to &lt;expiry&gt;)" (ADJ_PERIOD_INVALID)
+MSG-OP-243: "&lt;request no&gt; needs no quotation link" (ADJ_QUOTATION_NOT_REQUIRED)
+MSG-OP-244: "Enter the quotation number" (ADJ_QUOTATION_REF_REQUIRED)
+MSG-OP-245: "Enter the endorsement type, effective date and description" (ADJ_REQUEST_INCOMPLETE)
+MSG-OP-246: "Select the request type of a financial endorsement" (ADJ_REQUEST_TYPE_REQUIRED)
+MSG-OP-247: "&lt;invoice no&gt; is a return invoice: raise the request on the original" (ADJ_RETURN_INVOICE)
+MSG-OP-248: "Enter the increase or decrease of the total sum insured" (ADJ_TSI_CHANGE_REQUIRED)
+MSG-OP-249: "Endorsement type &lt;code&gt; has no class (FINANCIAL / NON_FINANCIAL)" (ADJ_TYPE_WITHOUT_CLASS)</t>
         </is>
       </c>
       <c r="M374" s="12" t="inlineStr">
@@ -41639,16 +41640,16 @@
       <c r="L375" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-256: "The invoice is paid: its payments are re-applied by Cashiering and the excess becomes an unapplied item."
-MSG-OP-257: "The new sum insured exceeds the package limit: Marketing prepares a quotation."
-MSG-OP-258: "A request is approved by someone who did not raise or validate it" (ADJ_FOUR_EYES)
-MSG-OP-259: "&lt;request no&gt; has not passed validation yet" (ADJ_NOT_VALIDATED)
-MSG-OP-260: "Internal adjustments have no endorsement slip" (ADJ_NO_SLIP_FOR_INTERNAL)
-MSG-OP-261: "Cumulative adjustments of &lt;to plain string&gt; exceed the baseline of &lt;to plain string&gt;% of the original premium &lt;to plain string&gt;: review the previous adjustments and give the justification to proceed" (ADJ_OVER_BASELINE)
-MSG-OP-262: "The TSI increase exceeds the package limit: link the quotation prepared by Marketing first" (ADJ_QUOTATION_REQUIRED)
-MSG-OP-263: "&lt;request no&gt; is &lt;stage&gt; and can no longer be changed" (ADJ_REQUEST_NOT_EDITABLE)
-MSG-OP-264: "&lt;request no&gt; is &lt;stage&gt;, not &lt;expected&gt;" (ADJ_WRONG_STAGE)
-MSG-OP-265: "Payments can only be re-applied once Cashiering is available; the request stays awaiting re-application" (PAYMENT_REAPPLIER_UNAVAILABLE)</t>
+MSG-OP-254: "The invoice is paid: its payments are re-applied by Cashiering and the excess becomes an unapplied item."
+MSG-OP-255: "The new sum insured exceeds the package limit: Marketing prepares a quotation."
+MSG-OP-256: "A request is approved by someone who did not raise or validate it" (ADJ_FOUR_EYES)
+MSG-OP-257: "&lt;request no&gt; has not passed validation yet" (ADJ_NOT_VALIDATED)
+MSG-OP-258: "Internal adjustments have no endorsement slip" (ADJ_NO_SLIP_FOR_INTERNAL)
+MSG-OP-259: "Cumulative adjustments of &lt;to plain string&gt; exceed the baseline of &lt;to plain string&gt;% of the original premium &lt;to plain string&gt;: review the previous adjustments and give the justification to proceed" (ADJ_OVER_BASELINE)
+MSG-OP-260: "The TSI increase exceeds the package limit: link the quotation prepared by Marketing first" (ADJ_QUOTATION_REQUIRED)
+MSG-OP-261: "&lt;request no&gt; is &lt;stage&gt; and can no longer be changed" (ADJ_REQUEST_NOT_EDITABLE)
+MSG-OP-262: "&lt;request no&gt; is &lt;stage&gt;, not &lt;expected&gt;" (ADJ_WRONG_STAGE)
+MSG-OP-263: "Payments can only be re-applied once Cashiering is available; the request stays awaiting re-application" (PAYMENT_REAPPLIER_UNAVAILABLE)</t>
         </is>
       </c>
       <c r="M375" s="12" t="inlineStr">
@@ -41723,8 +41724,8 @@
       <c r="L376" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-268: "Select the requests to post" (ADJ_BATCH_EMPTY)
-MSG-OP-269: "Select the return reason" (ADJ_RETURN_REASON_REQUIRED)</t>
+MSG-OP-266: "Select the requests to post" (ADJ_BATCH_EMPTY)
+MSG-OP-267: "Select the return reason" (ADJ_RETURN_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M376" s="12" t="inlineStr">
@@ -41799,8 +41800,8 @@
       <c r="L377" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-271: "&lt;invoice no&gt; has a balance of &lt;to plain string&gt;, outside the file range" (ADJ_BALANCE_OUT_OF_RANGE)
-MSG-OP-272: "&lt;invoice no&gt; has no premium receivable balance" (ADJ_NOTHING_TO_WRITE_OFF)</t>
+MSG-OP-269: "&lt;invoice no&gt; has a balance of &lt;to plain string&gt;, outside the file range" (ADJ_BALANCE_OUT_OF_RANGE)
+MSG-OP-270: "&lt;invoice no&gt; has no premium receivable balance" (ADJ_NOTHING_TO_WRITE_OFF)</t>
         </is>
       </c>
       <c r="M377" s="12" t="inlineStr">
@@ -41875,10 +41876,11 @@
       <c r="L378" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-275: "Enter valid e-mail addresses"
-MSG-OP-278: "Cycle &lt;cycle no&gt; is closed" (RECON_CYCLE_CLOSED)
-MSG-OP-279: "Pair a BDOI-only item with an insurer-only item of the same cycle" (RECON_PAIR_INVALID)
-MSG-OP-280: "Only a paired item can be split" (RECON_SPLIT_INVALID)</t>
+MSG-OP-272: "Enter valid e-mail addresses"
+MSG-OP-275: "Select the insurer"
+MSG-OP-276: "Cycle &lt;cycle no&gt; is closed" (RECON_CYCLE_CLOSED)
+MSG-OP-277: "Pair a BDOI-only item with an insurer-only item of the same cycle" (RECON_PAIR_INVALID)
+MSG-OP-278: "Only a paired item can be split" (RECON_SPLIT_INVALID)</t>
         </is>
       </c>
       <c r="M378" s="12" t="inlineStr">
@@ -41953,9 +41955,9 @@
       <c r="L379" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-282: "The booking period ends before it starts" (RECON_EXTRACT_PERIOD)
-MSG-OP-283: "No invoice was booked with &lt;insurer code&gt; from &lt;from&gt; to &lt;to&gt;" (RECON_NOTHING_TO_EXTRACT)
-MSG-OP-284: "Enter the insurer's e-mail address: &lt;insurer code&gt; has no placement e-mail in the catalog" (RECON_NO_RECIPIENT)</t>
+MSG-OP-280: "The booking period ends before it starts" (RECON_EXTRACT_PERIOD)
+MSG-OP-281: "No invoice was booked with &lt;insurer code&gt; from &lt;from&gt; to &lt;to&gt;" (RECON_NOTHING_TO_EXTRACT)
+MSG-OP-282: "Enter the insurer's e-mail address: &lt;insurer code&gt; has no placement e-mail in the catalog" (RECON_NO_RECIPIENT)</t>
         </is>
       </c>
       <c r="M379" s="12" t="inlineStr">
@@ -42030,13 +42032,13 @@
       <c r="L380" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-287: "Upload the production of &lt;insurer code&gt; from Production Reconciliation - Uploads (company not known)" (RECON_COMPANY_UNKNOWN)
-MSG-OP-288: "The file is not in the production register layout: column '&lt;wanted&gt;' missing" (RECON_FILE_LAYOUT)
-MSG-OP-289: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not an amount" (RECON_ROW_AMOUNT)
-MSG-OP-290: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not a date" (RECON_ROW_DATE)
-MSG-OP-291: "Row &lt;row no&gt; has neither invoice nor policy number" (RECON_ROW_INCOMPLETE)
-MSG-OP-292: "Row &lt;row no&gt; has no insurer or production month (yyyy-MM)" (RECON_ROW_INCOMPLETE)
-MSG-OP-293: "Upload refused: &lt;get&gt;" (RECON_UPLOAD_DUPLICATE)</t>
+MSG-OP-285: "Upload the production of &lt;insurer code&gt; from Production Reconciliation - Insurer Feedback (company not known)" (RECON_COMPANY_UNKNOWN)
+MSG-OP-286: "The file is not in the production register layout: column '&lt;wanted&gt;' missing" (RECON_FILE_LAYOUT)
+MSG-OP-287: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not an amount" (RECON_ROW_AMOUNT)
+MSG-OP-288: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not a date" (RECON_ROW_DATE)
+MSG-OP-289: "Row &lt;row no&gt; has neither invoice nor policy number" (RECON_ROW_INCOMPLETE)
+MSG-OP-290: "Row &lt;row no&gt; has no insurer or production month (yyyy-MM)" (RECON_ROW_INCOMPLETE)
+MSG-OP-291: "Upload refused: &lt;earlier upload&gt;" (RECON_UPLOAD_DUPLICATE)</t>
         </is>
       </c>
       <c r="M380" s="12" t="inlineStr">
@@ -42111,8 +42113,8 @@
       <c r="L381" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-298: "Extraction schedule already exists: &lt;key&gt;" (DUPLICATE)
-MSG-OP-299: "Choose the company and the insurer of the schedule" (RECON_SCHEDULE_INSURER)</t>
+MSG-OP-296: "Extraction schedule already exists: &lt;key&gt;" (DUPLICATE)
+MSG-OP-297: "Choose the company and the insurer of the schedule" (RECON_SCHEDULE_INSURER)</t>
         </is>
       </c>
       <c r="M381" s="12" t="inlineStr">
@@ -42187,15 +42189,15 @@
       <c r="L382" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-303: "Account &lt;invoice no&gt; is already &lt;tag&gt;" (DP_ITEM_STATE)
-MSG-OP-304: "No invoice of the list is booked: upload it from Commission Receivables" (DP_LIST_COMPANY)
-MSG-OP-305: "&lt;file name&gt; was already taken in as &lt;list no&gt;" (DP_LIST_DUPLICATE)
-MSG-OP-306: "The DP list has no 'Invoice No.' column" (DP_LIST_LAYOUT)
-MSG-OP-307: "Name the DP list &lt;Branch&gt;_DP_&lt;yyyyMMdd&gt; (e.g. HO_DP_20260930.xlsx): &lt;file name&gt;" (DP_LIST_NAME)
-MSG-OP-308: "The date in &lt;file name&gt; is not a date (yyyyMMdd)" (DP_LIST_NAME)
-MSG-OP-309: "The DP list was not taken in: &lt;null&gt;" (DP_LIST_REFUSED)
-MSG-OP-310: "The row has no invoice number" (DP_ROW_INCOMPLETE)
-MSG-OP-311: "Premium '&lt;premium&gt;' is not an amount" (DP_ROW_PREMIUM)</t>
+MSG-OP-301: "Account &lt;invoice no&gt; is already &lt;tag&gt;" (DP_ITEM_STATE)
+MSG-OP-302: "No invoice of the list is booked: upload it from Commission Receivables" (DP_LIST_COMPANY)
+MSG-OP-303: "&lt;file name&gt; was already taken in as &lt;list no&gt;" (DP_LIST_DUPLICATE)
+MSG-OP-304: "The DP list has no 'Invoice No.' column" (DP_LIST_LAYOUT)
+MSG-OP-305: "Name the DP list &lt;Branch&gt;_DP_&lt;yyyyMMdd&gt; (e.g. HO_DP_20260930.xlsx): &lt;file name&gt;" (DP_LIST_NAME)
+MSG-OP-306: "The date in &lt;file name&gt; is not a date (yyyyMMdd)" (DP_LIST_NAME)
+MSG-OP-307: "The DP list was not taken in: &lt;reason&gt;" (DP_LIST_REFUSED)
+MSG-OP-308: "The row has no invoice number" (DP_ROW_INCOMPLETE)
+MSG-OP-309: "Premium '&lt;premium&gt;' is not an amount" (DP_ROW_PREMIUM)</t>
         </is>
       </c>
       <c r="M382" s="12" t="inlineStr">
@@ -42270,8 +42272,8 @@
       <c r="L383" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-314: "Account &lt;invoice no&gt; is on a billing: cancel the billing first" (DP_ITEM_BILLED)
-MSG-OP-315: "Account &lt;invoice no&gt; (&lt;tag&gt;) cannot be &lt;action&gt;" (DP_ITEM_STATE)</t>
+MSG-OP-312: "Account &lt;invoice no&gt; is on a billing: cancel the billing first" (DP_ITEM_BILLED)
+MSG-OP-313: "Account &lt;invoice no&gt; (&lt;tag&gt;) cannot be &lt;action&gt;" (DP_ITEM_STATE)</t>
         </is>
       </c>
       <c r="M383" s="12" t="inlineStr">
@@ -42346,17 +42348,17 @@
       <c r="L384" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-318: "Choose the bank account the commission was received in" (DP_BANK_REQUIRED)
-MSG-OP-319: "Billing &lt;billing no&gt; has no approved account to collect" (DP_BILLING_NOT_APPROVED)
-MSG-OP-320: "Billing &lt;billing no&gt; is not waiting for the insurer" (DP_BILLING_NOT_AWAITING)
-MSG-OP-321: "Billing &lt;billing no&gt; was already sent" (DP_BILLING_SENT)
-MSG-OP-322: "Account &lt;invoice no&gt; is not confirmed for billing (&lt;tag&gt;)" (DP_ITEM_STATE)
-MSG-OP-323: "No account is confirmed for billing" (DP_NOTHING_TO_BILL)
-MSG-OP-324: "Invoice &lt;invoice no&gt; is not on billing &lt;billing no&gt;" (DP_NOT_ON_BILLING)
-MSG-OP-325: "Enter the e-mail address of &lt;insurer code&gt;" (DP_NO_RECIPIENT)
-MSG-OP-326: "Give the insurer's reason for rejecting &lt;invoice no&gt;" (DP_REASON_REQUIRED)
-MSG-OP-327: "Choose a direct payment reinstatement reason" (DP_REINSTATE_REASON)
-MSG-OP-328: "Invoice &lt;invoice no&gt; is not tagged direct payment by Marketing: its premium receivable cannot be reversed" (DP_TAG_INVALID)</t>
+MSG-OP-315: "Choose the bank account the commission was received in" (DP_BANK_REQUIRED)
+MSG-OP-316: "Billing &lt;billing no&gt; has no approved account to collect" (DP_BILLING_NOT_APPROVED)
+MSG-OP-317: "Billing &lt;billing no&gt; is not waiting for the insurer" (DP_BILLING_NOT_AWAITING)
+MSG-OP-318: "Billing &lt;billing no&gt; was already sent" (DP_BILLING_SENT)
+MSG-OP-319: "Account &lt;invoice no&gt; is not confirmed for billing (&lt;tag&gt;)" (DP_ITEM_STATE)
+MSG-OP-320: "No account is confirmed for billing" (DP_NOTHING_TO_BILL)
+MSG-OP-321: "Invoice &lt;invoice no&gt; is not on billing &lt;billing no&gt;" (DP_NOT_ON_BILLING)
+MSG-OP-322: "Enter the e-mail address of &lt;insurer code&gt;" (DP_NO_RECIPIENT)
+MSG-OP-323: "Give the insurer's reason for rejecting &lt;invoice no&gt;" (DP_REASON_REQUIRED)
+MSG-OP-324: "Choose a direct payment reinstatement reason" (DP_REINSTATE_REASON)
+MSG-OP-325: "Invoice &lt;invoice no&gt; is not tagged direct payment by Marketing: its premium receivable cannot be reversed" (DP_TAG_INVALID)</t>
         </is>
       </c>
       <c r="M384" s="12" t="inlineStr">
@@ -42431,9 +42433,9 @@
       <c r="L385" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-331: "Billing &lt;billing no&gt; does not exist" (DP_BILLING_UNKNOWN)
-MSG-OP-332: "Decision '&lt;decision&gt;' is neither APPROVED nor REJECTED" (DP_RESPONSE_DECISION)
-MSG-OP-333: "The insurer's answer has no '&lt;header&gt;' column" (DP_RESPONSE_LAYOUT)</t>
+MSG-OP-328: "Billing &lt;billing no&gt; does not exist" (DP_BILLING_UNKNOWN)
+MSG-OP-329: "Decision '&lt;decision&gt;' is not one of Approved or Rejected (or Yes / No)" (DP_RESPONSE_DECISION)
+MSG-OP-330: "The insurer's answer has no '&lt;header&gt;' column" (DP_RESPONSE_LAYOUT)</t>
         </is>
       </c>
       <c r="M385" s="12" t="inlineStr">
@@ -42508,10 +42510,10 @@
       <c r="L386" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-336: "Incentive scheme already exists: &lt;key&gt;" (DUPLICATE)
-MSG-OP-337: "The scheme ends before it starts" (INCENTIVE_SCHEME_DATES)
-MSG-OP-338: "Each tier needs a minimum basic premium and a fixed amount above zero" (INCENTIVE_TIER_INVALID)
-MSG-OP-339: "Each tier needs a production target and a rate above zero" (INCENTIVE_TIER_INVALID)</t>
+MSG-OP-333: "Incentive scheme already exists: &lt;key&gt;" (DUPLICATE)
+MSG-OP-334: "The scheme ends before it starts" (INCENTIVE_SCHEME_DATES)
+MSG-OP-335: "Each tier needs a minimum basic premium and a fixed amount above zero" (INCENTIVE_TIER_INVALID)
+MSG-OP-336: "Each tier needs a production target and a rate above zero" (INCENTIVE_TIER_INVALID)</t>
         </is>
       </c>
       <c r="M386" s="12" t="inlineStr">
@@ -42586,11 +42588,11 @@
       <c r="L387" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-341: "The company has no head office branch" (INCENTIVE_NO_HEAD_OFFICE)
-MSG-OP-342: "Run &lt;run no&gt; earned no incentive to post" (INCENTIVE_RUN_NOTHING)
-MSG-OP-343: "The period ends before it starts" (INCENTIVE_RUN_PERIOD)
-MSG-OP-344: "Run &lt;run no&gt; is &lt;status&gt; and cannot change" (INCENTIVE_RUN_STATE)
-MSG-OP-345: "Scheme &lt;name&gt; has no tiers yet (targets and amounts from BDOI)" (INCENTIVE_SCHEME_EMPTY)</t>
+MSG-OP-338: "The company has no head office branch" (INCENTIVE_NO_HEAD_OFFICE)
+MSG-OP-339: "Run &lt;run no&gt; earned no incentive to post" (INCENTIVE_RUN_NOTHING)
+MSG-OP-340: "The period ends before it starts" (INCENTIVE_RUN_PERIOD)
+MSG-OP-341: "Run &lt;run no&gt; is &lt;status&gt; and cannot change" (INCENTIVE_RUN_STATE)
+MSG-OP-342: "Scheme &lt;name&gt; has no tiers yet: add its targets and amounts first" (INCENTIVE_SCHEME_EMPTY)</t>
         </is>
       </c>
       <c r="M387" s="12" t="inlineStr">
@@ -42665,12 +42667,12 @@
       <c r="L388" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-348: "The tax withheld must be above zero" (CERT_AMOUNT)
-MSG-OP-349: "Choose the company and the insurer of the certificate" (CERT_INSURER_REQUIRED)
-MSG-OP-350: "Only a rejected submission can be resubmitted" (CERT_NOT_REJECTED)
-MSG-OP-351: "Tag the certificate to at least one official receipt" (CERT_NO_OR)
-MSG-OP-352: "The certificate period ends before it starts" (CERT_PERIOD)
-MSG-OP-353: "Give the reason of the rejection" (CERT_REASON_REQUIRED)</t>
+MSG-OP-345: "The tax withheld must be above zero" (CERT_AMOUNT)
+MSG-OP-346: "Choose the company and the insurer of the certificate" (CERT_INSURER_REQUIRED)
+MSG-OP-347: "Only a rejected submission can be resubmitted" (CERT_NOT_REJECTED)
+MSG-OP-348: "Tag the certificate to at least one official receipt" (CERT_NO_OR)
+MSG-OP-349: "The certificate period ends before it starts" (CERT_PERIOD)
+MSG-OP-350: "Give the reason of the rejection" (CERT_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M388" s="12" t="inlineStr">
@@ -42745,11 +42747,12 @@
       <c r="L389" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-355: "An active scheme needs at least one tier"
-MSG-OP-356: "Enter a period that ends after it starts"
-MSG-OP-357: "Record the insurer decision of at least one account"
-MSG-OP-358: "The scheme ends before it starts"
-MSG-OP-359: "The tax withheld must be above zero"</t>
+MSG-OP-352: "An active scheme needs at least one tier"
+MSG-OP-353: "Enter a period that ends after it starts"
+MSG-OP-354: "Record the insurer decision of at least one account"
+MSG-OP-355: "The scheme ends before it starts"
+MSG-OP-356: "The scheme name is required"
+MSG-OP-357: "The tax withheld must be above zero"</t>
         </is>
       </c>
       <c r="M389" s="12" t="inlineStr">
@@ -42824,8 +42827,8 @@
       <c r="L390" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-363: "Feed &lt;code&gt; is inactive" (FLOW_IN_FEED_INACTIVE)
-MSG-OP-364: "No module processes uploads of feed &lt;feed code&gt; yet" (FLOW_IN_NO_HANDLER)</t>
+MSG-OP-361: "Feed &lt;code&gt; is inactive" (FLOW_IN_FEED_INACTIVE)
+MSG-OP-362: "No module processes uploads of feed &lt;feed code&gt; yet" (FLOW_IN_NO_HANDLER)</t>
         </is>
       </c>
       <c r="M390" s="12" t="inlineStr">
@@ -42888,9 +42891,9 @@
       <c r="L391" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-366: "Prefix is required"
-MSG-OP-368: "The range must end at or after its start"
-MSG-OP-369: "The series becomes active for issuing receipts."</t>
+MSG-OP-364: "Prefix is required"
+MSG-OP-366: "The range must end at or after its start"
+MSG-OP-367: "The series becomes active for issuing receipts."</t>
         </is>
       </c>
       <c r="M391" s="12" t="inlineStr">
@@ -42953,8 +42956,8 @@
       <c r="L392" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-370: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-OP-371: "&lt;Column&gt; is mandatory"</t>
+MSG-OP-368: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-OP-369: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M392" s="12" t="inlineStr">
@@ -43017,8 +43020,8 @@
       <c r="L393" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-372: "A certificate tag needs the certificate number"
-MSG-OP-373: "Path must be CASH or CERTIFICATE"</t>
+MSG-OP-370: "A certificate tag needs the certificate number"
+MSG-OP-371: "Path must be CASH or CERTIFICATE"</t>
         </is>
       </c>
       <c r="M393" s="12" t="inlineStr">
@@ -43081,7 +43084,7 @@
       <c r="L394" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-374: "Possible duplicate of &lt;preview&gt;"</t>
+MSG-OP-372: "Possible duplicate of &lt;preview&gt;"</t>
         </is>
       </c>
       <c r="M394" s="12" t="inlineStr">
@@ -43144,7 +43147,7 @@
       <c r="L395" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-375: "The amount must be above zero"</t>
+MSG-OP-373: "The amount must be above zero"</t>
         </is>
       </c>
       <c r="M395" s="12" t="inlineStr">
@@ -43207,7 +43210,7 @@
       <c r="L396" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-376: "The basic commission must be above zero"</t>
+MSG-OP-374: "The basic commission must be above zero"</t>
         </is>
       </c>
       <c r="M396" s="12" t="inlineStr">
@@ -43270,13 +43273,13 @@
       <c r="L397" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-377: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-OP-378: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-OP-379: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-OP-380: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-OP-381: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-OP-382: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-OP-383: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-OP-375: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-OP-376: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-OP-377: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-OP-378: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-OP-379: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-OP-380: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-OP-381: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M397" s="12" t="inlineStr">
@@ -54411,7 +54414,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>ARN-2026-940001 (Motor; booking and endorsement invoices paid in full; booking invoice remitted with the insurer OR), ARN-2026-940002 (Property; requests at every adjustment stage; gross premium differs in the insurer register), ARN-2026-940003 (direct payment), ARN-2026-940004 (CGL; partly paid; hold request waiting; flat cancellation ready for posting)</t>
+          <t>ARN-2026-940001 (Motor; booking and endorsement invoices paid in full; booking invoice remitted with the insurer OR), ARN-2026-940002 (Property; requests at every adjustment stage; gross premium differs in the insurer register), ARN-2026-940003 (direct payment), ARN-2026-940004 (CGL; partly paid; flat cancellation ready for posting), ARN-2026-940008 (Motor; hold request waiting)</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -54461,7 +54464,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>A remitted batch of ARN-2026-940001 with its insurer OR; a batch in review with the endorsement invoice; a hold request of ARN-2026-940004 waiting for approval; a special remittance request; incentive rule INS-MGIC Property CBG 2 % within 30 days of inception</t>
+          <t>A remitted batch of ARN-2026-940001 with its insurer OR; a batch in review with the endorsement invoice; a hold request of ARN-2026-940008 waiting for approval; a special remittance request; incentive rule INS-MGIC Property CBG 2 % within 30 days of inception</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Deliverable builders take the client logo from the theme pack and the platform logo from its new folder; BRD-02 set rebuilt on the merged texts
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-02_Operations/04_BIBS_TestPlan_BRD-02_Operations_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-02_Operations/04_BIBS_TestPlan_BRD-02_Operations_v2.0.xlsx
@@ -13371,7 +13371,7 @@
       <c r="L7" s="12" t="inlineStr">
         <is>
           <t>The account is locked at the third failure; the System Administrator unlocks it in Administration &gt; Users.
-Message "Account is locked. Contact your administrator." (AUTHENTICATION_FAILED).</t>
+Message "Invalid user name or password" (AUTHENTICATION_FAILED).</t>
         </is>
       </c>
       <c r="M7" s="12" t="inlineStr">
@@ -29308,7 +29308,7 @@
       <c r="L217" s="12" t="inlineStr">
         <is>
           <t>Refused.
-Message "Pair a BDOI-only item with an insurer-only item of the same cycle" (RECON_PAIR_INVALID).</t>
+Message "Pair a booked-only item with an insurer-only item of the same cycle" (RECON_PAIR_INVALID).</t>
         </is>
       </c>
       <c r="M217" s="12" t="inlineStr">
@@ -41059,12 +41059,13 @@
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
 MSG-OP-174: "The file must have the columns &lt;details&gt;" (FEED_FILE_COLUMNS)
 MSG-OP-175: "The file has no lines" (FEED_FILE_EMPTY)
-MSG-OP-176: "Line &lt;line no&gt;: &lt;column&gt; must be a date such as 28-Oct-2026" (FEED_VALUE_INVALID)
-MSG-OP-177: "Line &lt;line no&gt;: &lt;column&gt; must be an amount" (FEED_VALUE_INVALID)
-MSG-OP-178: "Line &lt;line no&gt;: &lt;column&gt; is missing" (FEED_VALUE_MISSING)
-MSG-OP-179: "Batch &lt;batch no&gt; is &lt;stage&gt;: not yet approved" (REMIT_OR_BATCH_STAGE)
-MSG-OP-180: "OR &lt;number&gt; was already recorded for client &lt;client code&gt;" (REMIT_OR_DUPLICATE)
-MSG-OP-181: "Invoice &lt;invoice no&gt; was excluded from &lt;batch no&gt;" (REMIT_OR_LINE_EXCLUDED)</t>
+MSG-OP-176: "The file is not a readable Excel workbook" (FEED_FILE_UNREADABLE)
+MSG-OP-177: "Line &lt;line no&gt;: &lt;column&gt; must be a date such as 28-Oct-2026" (FEED_VALUE_INVALID)
+MSG-OP-178: "Line &lt;line no&gt;: &lt;column&gt; must be an amount" (FEED_VALUE_INVALID)
+MSG-OP-179: "Line &lt;line no&gt;: &lt;column&gt; is missing" (FEED_VALUE_MISSING)
+MSG-OP-180: "Batch &lt;batch no&gt; is &lt;stage&gt;: not yet approved" (REMIT_OR_BATCH_STAGE)
+MSG-OP-181: "OR &lt;number&gt; was already recorded for client &lt;client code&gt;" (REMIT_OR_DUPLICATE)
+MSG-OP-182: "Invoice &lt;invoice no&gt; was excluded from &lt;batch no&gt;" (REMIT_OR_LINE_EXCLUDED)</t>
         </is>
       </c>
       <c r="M368" s="12" t="inlineStr">
@@ -41139,15 +41140,15 @@
       <c r="L369" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-183: "&lt;processor&gt; is not an active remittance processor" (HOLD_ASSIGNEE_NOT_ELIGIBLE)
-MSG-OP-184: "The hold-until date must be in the future" (HOLD_DATE)
-MSG-OP-185: "Invoice &lt;invoice no&gt; already has hold &lt;request no&gt;" (HOLD_DUPLICATE)
-MSG-OP-186: "The extension must be later than &lt;hold until&gt;" (HOLD_EXTENSION_DATE)
-MSG-OP-187: "Hold &lt;request no&gt; must be approved by another user" (HOLD_FOUR_EYES)
-MSG-OP-188: "Hold &lt;request no&gt; must be decided by another user" (HOLD_FOUR_EYES)
-MSG-OP-189: "Invoice &lt;invoice no&gt; cannot be held: remittance status &lt;remittance status&gt;" (HOLD_INVOICE_NOT_HOLDABLE)
-MSG-OP-190: "Hold &lt;request no&gt; is &lt;stage&gt;, not &lt;stage&gt;" (HOLD_STAGE)
-MSG-OP-191: "Hold &lt;request no&gt; is not active" (HOLD_STAGE)</t>
+MSG-OP-184: "&lt;processor&gt; is not an active remittance processor" (HOLD_ASSIGNEE_NOT_ELIGIBLE)
+MSG-OP-185: "The hold-until date must be in the future" (HOLD_DATE)
+MSG-OP-186: "Invoice &lt;invoice no&gt; already has hold &lt;request no&gt;" (HOLD_DUPLICATE)
+MSG-OP-187: "The extension must be later than &lt;hold until&gt;" (HOLD_EXTENSION_DATE)
+MSG-OP-188: "Hold &lt;request no&gt; must be approved by another user" (HOLD_FOUR_EYES)
+MSG-OP-189: "Hold &lt;request no&gt; must be decided by another user" (HOLD_FOUR_EYES)
+MSG-OP-190: "Invoice &lt;invoice no&gt; cannot be held: remittance status &lt;remittance status&gt;" (HOLD_INVOICE_NOT_HOLDABLE)
+MSG-OP-191: "Hold &lt;request no&gt; is &lt;stage&gt;, not &lt;stage&gt;" (HOLD_STAGE)
+MSG-OP-192: "Hold &lt;request no&gt; is not active" (HOLD_STAGE)</t>
         </is>
       </c>
       <c r="M369" s="12" t="inlineStr">
@@ -41222,9 +41223,9 @@
       <c r="L370" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-193: "Invoice &lt;invoice no&gt; already has request &lt;request no&gt;" (SPECIAL_REMIT_DUPLICATE)
-MSG-OP-194: "Request &lt;request no&gt; must be approved by another user" (SPECIAL_REMIT_FOUR_EYES)
-MSG-OP-195: "Invoice &lt;invoice no&gt; cannot be remitted specially: &lt;why&gt;" (SPECIAL_REMIT_NOT_ELIGIBLE)</t>
+MSG-OP-194: "Invoice &lt;invoice no&gt; already has request &lt;request no&gt;" (SPECIAL_REMIT_DUPLICATE)
+MSG-OP-195: "Request &lt;request no&gt; must be approved by another user" (SPECIAL_REMIT_FOUR_EYES)
+MSG-OP-196: "Invoice &lt;invoice no&gt; cannot be remitted specially: &lt;why&gt;" (SPECIAL_REMIT_NOT_ELIGIBLE)</t>
         </is>
       </c>
       <c r="M370" s="12" t="inlineStr">
@@ -41299,17 +41300,17 @@
       <c r="L371" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-198: "Choose the currency"
-MSG-OP-199: "Choose what the deduction settles"
-MSG-OP-200: "Enter a positive amount with at most 2 decimals"
-MSG-OP-203: "Select the insurer"
-MSG-OP-204: "Source reference is required"
-MSG-OP-205: "The confirmation date cannot be in the future"
-MSG-OP-206: "Select the company" (COMPANY_REQUIRED)
-MSG-OP-207: "A deduction needs a positive amount" (REMIT_DEDUCTION_AMOUNT)
-MSG-OP-208: "Deduction &lt;deduction no&gt; must be confirmed by another user" (REMIT_DEDUCTION_FOUR_EYES)
-MSG-OP-209: "Deduction &lt;deduction no&gt; can only change as a draft" (REMIT_DEDUCTION_STAGE)
-MSG-OP-210: "Deduction &lt;deduction no&gt; needs the insurer's confirmation reference and date before submission" (REMIT_DEDUCTION_UNCONFIRMED)</t>
+MSG-OP-199: "Choose the currency"
+MSG-OP-200: "Choose what the deduction settles"
+MSG-OP-201: "Enter a positive amount with at most 2 decimals"
+MSG-OP-204: "Select the insurer"
+MSG-OP-205: "Source reference is required"
+MSG-OP-206: "The confirmation date cannot be in the future"
+MSG-OP-207: "Select the company" (COMPANY_REQUIRED)
+MSG-OP-208: "A deduction needs a positive amount" (REMIT_DEDUCTION_AMOUNT)
+MSG-OP-209: "Deduction &lt;deduction no&gt; must be confirmed by another user" (REMIT_DEDUCTION_FOUR_EYES)
+MSG-OP-210: "Deduction &lt;deduction no&gt; can only change as a draft" (REMIT_DEDUCTION_STAGE)
+MSG-OP-211: "Deduction &lt;deduction no&gt; needs the insurer's confirmation reference and date before submission" (REMIT_DEDUCTION_UNCONFIRMED)</t>
         </is>
       </c>
       <c r="M371" s="12" t="inlineStr">
@@ -41384,12 +41385,12 @@
       <c r="L372" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-212: "Rate must be above 0 and at most 100"
-MSG-OP-213: "Select the insurer"
-MSG-OP-214: "The rule cannot end before it starts"
-MSG-OP-215: "Window must be 1 to 366 days"
-MSG-OP-216: "Choose the company of the rule" (COMPANY_REQUIRED)
-MSG-OP-217: "The rule cannot end before it starts" (INCENTIVE_RULE_PERIOD)</t>
+MSG-OP-213: "Rate must be above 0 and at most 100"
+MSG-OP-214: "Select the insurer"
+MSG-OP-215: "The rule cannot end before it starts"
+MSG-OP-216: "Window must be 1 to 366 days"
+MSG-OP-217: "Choose the company of the rule" (COMPANY_REQUIRED)
+MSG-OP-218: "The rule cannot end before it starts" (INCENTIVE_RULE_PERIOD)</t>
         </is>
       </c>
       <c r="M372" s="12" t="inlineStr">
@@ -41464,9 +41465,9 @@
       <c r="L373" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-219: "A payment request needs a positive amount" (DISBURSEMENT_AMOUNT)
-MSG-OP-220: "Too many references on one payment request" (DISBURSEMENT_REFERENCES)
-MSG-OP-221: "Payment request &lt;request no&gt; is &lt;status&gt; and cannot be &lt;action&gt;" (DISBURSEMENT_STATUS)</t>
+MSG-OP-220: "A payment request needs a positive amount" (DISBURSEMENT_AMOUNT)
+MSG-OP-221: "Too many references on one payment request" (DISBURSEMENT_REFERENCES)
+MSG-OP-222: "Payment request &lt;request no&gt; is &lt;status&gt; and cannot be &lt;action&gt;" (DISBURSEMENT_STATUS)</t>
         </is>
       </c>
       <c r="M373" s="12" t="inlineStr">
@@ -41541,31 +41542,31 @@
       <c r="L374" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-223: "A financial endorsement needs its request type"
-MSG-OP-225: "Describe the change"
-MSG-OP-226: "Enter at least one premium, charge or commission change"
-MSG-OP-227: "Enter the effective date"
-MSG-OP-228: "Enter the increase (positive) or decrease (negative)"
-MSG-OP-230: "Select the endorsement type"
-MSG-OP-231: "Select the reason for cancellation"
-MSG-OP-232: "The new expiry must be after the new inception"
-MSG-OP-233: "Enter the premium, charges or commission change" (ADJ_AMOUNTS_REQUIRED)
-MSG-OP-234: "Select the reason for cancellation" (ADJ_CANCELLATION_REASON_REQUIRED)
-MSG-OP-235: "Possible duplicate of &lt;details&gt; (same invoice, request type, reason and endorsement reference): give the justification to proceed" (ADJ_DUPLICATE_REQUEST)
-MSG-OP-236: "The effective date must be within the cover &lt;inception&gt; to &lt;expiry&gt;" (ADJ_EFFECTIVE_DATE_OUTSIDE_TERM)
-MSG-OP-237: "Request &lt;request no&gt; (&lt;&gt;) is still open on &lt;invoice no&gt;: a cancellation cannot be combined with another financial change" (ADJ_INCOMPATIBLE_REQUEST)
-MSG-OP-238: "Select at least one invoice" (ADJ_INVOICES_REQUIRED)
-MSG-OP-239: "Select between 1 and 50 invoices" (ADJ_INVOICES_REQUIRED)
-MSG-OP-240: "&lt;invoice no&gt; is cancelled or written off" (ADJ_INVOICE_CLOSED)
-MSG-OP-241: "A non-financial endorsement carries no request type, sum insured or amount change" (ADJ_NON_FINANCIAL_WITH_AMOUNTS)
-MSG-OP-242: "Enter a valid new period (a change of period keeps the term of &lt;inception&gt; to &lt;expiry&gt;)" (ADJ_PERIOD_INVALID)
-MSG-OP-243: "&lt;request no&gt; needs no quotation link" (ADJ_QUOTATION_NOT_REQUIRED)
-MSG-OP-244: "Enter the quotation number" (ADJ_QUOTATION_REF_REQUIRED)
-MSG-OP-245: "Enter the endorsement type, effective date and description" (ADJ_REQUEST_INCOMPLETE)
-MSG-OP-246: "Select the request type of a financial endorsement" (ADJ_REQUEST_TYPE_REQUIRED)
-MSG-OP-247: "&lt;invoice no&gt; is a return invoice: raise the request on the original" (ADJ_RETURN_INVOICE)
-MSG-OP-248: "Enter the increase or decrease of the total sum insured" (ADJ_TSI_CHANGE_REQUIRED)
-MSG-OP-249: "Endorsement type &lt;code&gt; has no class (FINANCIAL / NON_FINANCIAL)" (ADJ_TYPE_WITHOUT_CLASS)</t>
+MSG-OP-224: "A financial endorsement needs its request type"
+MSG-OP-226: "Describe the change"
+MSG-OP-227: "Enter at least one premium, charge or commission change"
+MSG-OP-228: "Enter the effective date"
+MSG-OP-229: "Enter the increase (positive) or decrease (negative)"
+MSG-OP-231: "Select the endorsement type"
+MSG-OP-232: "Select the reason for cancellation"
+MSG-OP-233: "The new expiry must be after the new inception"
+MSG-OP-234: "Enter the premium, charges or commission change" (ADJ_AMOUNTS_REQUIRED)
+MSG-OP-235: "Select the reason for cancellation" (ADJ_CANCELLATION_REASON_REQUIRED)
+MSG-OP-236: "Possible duplicate of &lt;details&gt; (same invoice, request type, reason and endorsement reference): give the justification to proceed" (ADJ_DUPLICATE_REQUEST)
+MSG-OP-237: "The effective date must be within the cover &lt;inception&gt; to &lt;expiry&gt;" (ADJ_EFFECTIVE_DATE_OUTSIDE_TERM)
+MSG-OP-238: "Request &lt;request no&gt; (&lt;&gt;) is still open on &lt;invoice no&gt;: a cancellation cannot be combined with another financial change" (ADJ_INCOMPATIBLE_REQUEST)
+MSG-OP-239: "Select at least one invoice" (ADJ_INVOICES_REQUIRED)
+MSG-OP-240: "Select between 1 and 50 invoices" (ADJ_INVOICES_REQUIRED)
+MSG-OP-241: "&lt;invoice no&gt; is cancelled or written off" (ADJ_INVOICE_CLOSED)
+MSG-OP-242: "A non-financial endorsement carries no request type, sum insured or amount change" (ADJ_NON_FINANCIAL_WITH_AMOUNTS)
+MSG-OP-243: "Enter a valid new period (a change of period keeps the term of &lt;inception&gt; to &lt;expiry&gt;)" (ADJ_PERIOD_INVALID)
+MSG-OP-244: "&lt;request no&gt; needs no quotation link" (ADJ_QUOTATION_NOT_REQUIRED)
+MSG-OP-245: "Enter the quotation number" (ADJ_QUOTATION_REF_REQUIRED)
+MSG-OP-246: "Enter the endorsement type, effective date and description" (ADJ_REQUEST_INCOMPLETE)
+MSG-OP-247: "Select the request type of a financial endorsement" (ADJ_REQUEST_TYPE_REQUIRED)
+MSG-OP-248: "&lt;invoice no&gt; is a return invoice: raise the request on the original" (ADJ_RETURN_INVOICE)
+MSG-OP-249: "Enter the increase or decrease of the total sum insured" (ADJ_TSI_CHANGE_REQUIRED)
+MSG-OP-250: "Endorsement type &lt;code&gt; has no class (FINANCIAL / NON_FINANCIAL)" (ADJ_TYPE_WITHOUT_CLASS)</t>
         </is>
       </c>
       <c r="M374" s="12" t="inlineStr">
@@ -41640,16 +41641,16 @@
       <c r="L375" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-254: "The invoice is paid: its payments are re-applied by Cashiering and the excess becomes an unapplied item."
-MSG-OP-255: "The new sum insured exceeds the package limit: Marketing prepares a quotation."
-MSG-OP-256: "A request is approved by someone who did not raise or validate it" (ADJ_FOUR_EYES)
-MSG-OP-257: "&lt;request no&gt; has not passed validation yet" (ADJ_NOT_VALIDATED)
-MSG-OP-258: "Internal adjustments have no endorsement slip" (ADJ_NO_SLIP_FOR_INTERNAL)
-MSG-OP-259: "Cumulative adjustments of &lt;to plain string&gt; exceed the baseline of &lt;to plain string&gt;% of the original premium &lt;to plain string&gt;: review the previous adjustments and give the justification to proceed" (ADJ_OVER_BASELINE)
-MSG-OP-260: "The TSI increase exceeds the package limit: link the quotation prepared by Marketing first" (ADJ_QUOTATION_REQUIRED)
-MSG-OP-261: "&lt;request no&gt; is &lt;stage&gt; and can no longer be changed" (ADJ_REQUEST_NOT_EDITABLE)
-MSG-OP-262: "&lt;request no&gt; is &lt;stage&gt;, not &lt;expected&gt;" (ADJ_WRONG_STAGE)
-MSG-OP-263: "Payments can only be re-applied once Cashiering is available; the request stays awaiting re-application" (PAYMENT_REAPPLIER_UNAVAILABLE)</t>
+MSG-OP-255: "The invoice is paid: its payments are re-applied by Cashiering and the excess becomes an unapplied item."
+MSG-OP-256: "The new sum insured exceeds the package limit: Marketing prepares a quotation."
+MSG-OP-257: "A request is approved by someone who did not raise or validate it" (ADJ_FOUR_EYES)
+MSG-OP-258: "&lt;request no&gt; has not passed validation yet" (ADJ_NOT_VALIDATED)
+MSG-OP-259: "Internal adjustments have no endorsement slip" (ADJ_NO_SLIP_FOR_INTERNAL)
+MSG-OP-260: "Cumulative adjustments of &lt;to plain string&gt; exceed the baseline of &lt;to plain string&gt;% of the original premium &lt;to plain string&gt;: review the previous adjustments and give the justification to proceed" (ADJ_OVER_BASELINE)
+MSG-OP-261: "The TSI increase exceeds the package limit: link the quotation prepared by Marketing first" (ADJ_QUOTATION_REQUIRED)
+MSG-OP-262: "&lt;request no&gt; is &lt;stage&gt; and can no longer be changed" (ADJ_REQUEST_NOT_EDITABLE)
+MSG-OP-263: "&lt;request no&gt; is &lt;stage&gt;, not &lt;expected&gt;" (ADJ_WRONG_STAGE)
+MSG-OP-264: "Payments can only be re-applied once Cashiering is available; the request stays awaiting re-application" (PAYMENT_REAPPLIER_UNAVAILABLE)</t>
         </is>
       </c>
       <c r="M375" s="12" t="inlineStr">
@@ -41724,8 +41725,8 @@
       <c r="L376" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-266: "Select the requests to post" (ADJ_BATCH_EMPTY)
-MSG-OP-267: "Select the return reason" (ADJ_RETURN_REASON_REQUIRED)</t>
+MSG-OP-267: "Select the requests to post" (ADJ_BATCH_EMPTY)
+MSG-OP-268: "Select the return reason" (ADJ_RETURN_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M376" s="12" t="inlineStr">
@@ -41800,8 +41801,8 @@
       <c r="L377" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-269: "&lt;invoice no&gt; has a balance of &lt;to plain string&gt;, outside the file range" (ADJ_BALANCE_OUT_OF_RANGE)
-MSG-OP-270: "&lt;invoice no&gt; has no premium receivable balance" (ADJ_NOTHING_TO_WRITE_OFF)</t>
+MSG-OP-270: "&lt;invoice no&gt; has a balance of &lt;to plain string&gt;, outside the file range" (ADJ_BALANCE_OUT_OF_RANGE)
+MSG-OP-271: "&lt;invoice no&gt; has no premium receivable balance" (ADJ_NOTHING_TO_WRITE_OFF)</t>
         </is>
       </c>
       <c r="M377" s="12" t="inlineStr">
@@ -41876,11 +41877,11 @@
       <c r="L378" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-272: "Enter valid e-mail addresses"
-MSG-OP-275: "Select the insurer"
-MSG-OP-276: "Cycle &lt;cycle no&gt; is closed" (RECON_CYCLE_CLOSED)
-MSG-OP-277: "Pair a BDOI-only item with an insurer-only item of the same cycle" (RECON_PAIR_INVALID)
-MSG-OP-278: "Only a paired item can be split" (RECON_SPLIT_INVALID)</t>
+MSG-OP-273: "Enter valid e-mail addresses"
+MSG-OP-276: "Select the insurer"
+MSG-OP-277: "Cycle &lt;cycle no&gt; is closed" (RECON_CYCLE_CLOSED)
+MSG-OP-278: "Pair a booked-only item with an insurer-only item of the same cycle" (RECON_PAIR_INVALID)
+MSG-OP-279: "Only a paired item can be split" (RECON_SPLIT_INVALID)</t>
         </is>
       </c>
       <c r="M378" s="12" t="inlineStr">
@@ -41955,9 +41956,9 @@
       <c r="L379" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-280: "The booking period ends before it starts" (RECON_EXTRACT_PERIOD)
-MSG-OP-281: "No invoice was booked with &lt;insurer code&gt; from &lt;from&gt; to &lt;to&gt;" (RECON_NOTHING_TO_EXTRACT)
-MSG-OP-282: "Enter the insurer's e-mail address: &lt;insurer code&gt; has no placement e-mail in the catalog" (RECON_NO_RECIPIENT)</t>
+MSG-OP-281: "The booking period ends before it starts" (RECON_EXTRACT_PERIOD)
+MSG-OP-282: "No invoice was booked with &lt;insurer code&gt; from &lt;from&gt; to &lt;to&gt;" (RECON_NOTHING_TO_EXTRACT)
+MSG-OP-283: "Enter the insurer's e-mail address: &lt;insurer code&gt; has no placement e-mail in the catalog" (RECON_NO_RECIPIENT)</t>
         </is>
       </c>
       <c r="M379" s="12" t="inlineStr">
@@ -42032,13 +42033,13 @@
       <c r="L380" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-285: "Upload the production of &lt;insurer code&gt; from Production Reconciliation - Insurer Feedback (company not known)" (RECON_COMPANY_UNKNOWN)
-MSG-OP-286: "The file is not in the production register layout: column '&lt;wanted&gt;' missing" (RECON_FILE_LAYOUT)
-MSG-OP-287: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not an amount" (RECON_ROW_AMOUNT)
-MSG-OP-288: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not a date" (RECON_ROW_DATE)
-MSG-OP-289: "Row &lt;row no&gt; has neither invoice nor policy number" (RECON_ROW_INCOMPLETE)
-MSG-OP-290: "Row &lt;row no&gt; has no insurer or production month (yyyy-MM)" (RECON_ROW_INCOMPLETE)
-MSG-OP-291: "Upload refused: &lt;earlier upload&gt;" (RECON_UPLOAD_DUPLICATE)</t>
+MSG-OP-286: "Upload the production of &lt;insurer code&gt; from Production Reconciliation - Insurer Feedback (company not known)" (RECON_COMPANY_UNKNOWN)
+MSG-OP-287: "The file is not in the production register layout: column '&lt;wanted&gt;' missing" (RECON_FILE_LAYOUT)
+MSG-OP-288: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not an amount" (RECON_ROW_AMOUNT)
+MSG-OP-289: "Row &lt;row no&gt;: &lt;header&gt; '&lt;v&gt;' is not a date" (RECON_ROW_DATE)
+MSG-OP-290: "Row &lt;row no&gt; has neither invoice nor policy number" (RECON_ROW_INCOMPLETE)
+MSG-OP-291: "Row &lt;row no&gt; has no insurer or production month (yyyy-MM)" (RECON_ROW_INCOMPLETE)
+MSG-OP-292: "Upload refused: &lt;earlier upload&gt;" (RECON_UPLOAD_DUPLICATE)</t>
         </is>
       </c>
       <c r="M380" s="12" t="inlineStr">
@@ -42113,8 +42114,8 @@
       <c r="L381" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-296: "Extraction schedule already exists: &lt;key&gt;" (DUPLICATE)
-MSG-OP-297: "Choose the company and the insurer of the schedule" (RECON_SCHEDULE_INSURER)</t>
+MSG-OP-297: "Extraction schedule already exists: &lt;key&gt;" (DUPLICATE)
+MSG-OP-298: "Choose the company and the insurer of the schedule" (RECON_SCHEDULE_INSURER)</t>
         </is>
       </c>
       <c r="M381" s="12" t="inlineStr">
@@ -42189,15 +42190,15 @@
       <c r="L382" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-301: "Account &lt;invoice no&gt; is already &lt;tag&gt;" (DP_ITEM_STATE)
-MSG-OP-302: "No invoice of the list is booked: upload it from Commission Receivables" (DP_LIST_COMPANY)
-MSG-OP-303: "&lt;file name&gt; was already taken in as &lt;list no&gt;" (DP_LIST_DUPLICATE)
-MSG-OP-304: "The DP list has no 'Invoice No.' column" (DP_LIST_LAYOUT)
-MSG-OP-305: "Name the DP list &lt;Branch&gt;_DP_&lt;yyyyMMdd&gt; (e.g. HO_DP_20260930.xlsx): &lt;file name&gt;" (DP_LIST_NAME)
-MSG-OP-306: "The date in &lt;file name&gt; is not a date (yyyyMMdd)" (DP_LIST_NAME)
-MSG-OP-307: "The DP list was not taken in: &lt;reason&gt;" (DP_LIST_REFUSED)
-MSG-OP-308: "The row has no invoice number" (DP_ROW_INCOMPLETE)
-MSG-OP-309: "Premium '&lt;premium&gt;' is not an amount" (DP_ROW_PREMIUM)</t>
+MSG-OP-302: "Account &lt;invoice no&gt; is already &lt;tag&gt;" (DP_ITEM_STATE)
+MSG-OP-303: "No invoice of the list is booked: upload it from Commission Receivables" (DP_LIST_COMPANY)
+MSG-OP-304: "&lt;file name&gt; was already taken in as &lt;list no&gt;" (DP_LIST_DUPLICATE)
+MSG-OP-305: "The DP list has no 'Invoice No.' column" (DP_LIST_LAYOUT)
+MSG-OP-306: "Name the DP list &lt;Branch&gt;_DP_&lt;yyyyMMdd&gt; (e.g. MAIN_DP_20260930.xlsx): &lt;file name&gt;" (DP_LIST_NAME)
+MSG-OP-307: "The date in &lt;file name&gt; is not a date (yyyyMMdd)" (DP_LIST_NAME)
+MSG-OP-308: "The DP list was not taken in: &lt;reason&gt;" (DP_LIST_REFUSED)
+MSG-OP-309: "The row has no invoice number" (DP_ROW_INCOMPLETE)
+MSG-OP-310: "Premium '&lt;premium&gt;' is not an amount" (DP_ROW_PREMIUM)</t>
         </is>
       </c>
       <c r="M382" s="12" t="inlineStr">
@@ -42272,8 +42273,8 @@
       <c r="L383" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-312: "Account &lt;invoice no&gt; is on a billing: cancel the billing first" (DP_ITEM_BILLED)
-MSG-OP-313: "Account &lt;invoice no&gt; (&lt;tag&gt;) cannot be &lt;action&gt;" (DP_ITEM_STATE)</t>
+MSG-OP-313: "Account &lt;invoice no&gt; is on a billing: cancel the billing first" (DP_ITEM_BILLED)
+MSG-OP-314: "Account &lt;invoice no&gt; (&lt;tag&gt;) cannot be &lt;action&gt;" (DP_ITEM_STATE)</t>
         </is>
       </c>
       <c r="M383" s="12" t="inlineStr">
@@ -42348,17 +42349,17 @@
       <c r="L384" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-315: "Choose the bank account the commission was received in" (DP_BANK_REQUIRED)
-MSG-OP-316: "Billing &lt;billing no&gt; has no approved account to collect" (DP_BILLING_NOT_APPROVED)
-MSG-OP-317: "Billing &lt;billing no&gt; is not waiting for the insurer" (DP_BILLING_NOT_AWAITING)
-MSG-OP-318: "Billing &lt;billing no&gt; was already sent" (DP_BILLING_SENT)
-MSG-OP-319: "Account &lt;invoice no&gt; is not confirmed for billing (&lt;tag&gt;)" (DP_ITEM_STATE)
-MSG-OP-320: "No account is confirmed for billing" (DP_NOTHING_TO_BILL)
-MSG-OP-321: "Invoice &lt;invoice no&gt; is not on billing &lt;billing no&gt;" (DP_NOT_ON_BILLING)
-MSG-OP-322: "Enter the e-mail address of &lt;insurer code&gt;" (DP_NO_RECIPIENT)
-MSG-OP-323: "Give the insurer's reason for rejecting &lt;invoice no&gt;" (DP_REASON_REQUIRED)
-MSG-OP-324: "Choose a direct payment reinstatement reason" (DP_REINSTATE_REASON)
-MSG-OP-325: "Invoice &lt;invoice no&gt; is not tagged direct payment by Marketing: its premium receivable cannot be reversed" (DP_TAG_INVALID)</t>
+MSG-OP-316: "Choose the bank account the commission was received in" (DP_BANK_REQUIRED)
+MSG-OP-317: "Billing &lt;billing no&gt; has no approved account to collect" (DP_BILLING_NOT_APPROVED)
+MSG-OP-318: "Billing &lt;billing no&gt; is not waiting for the insurer" (DP_BILLING_NOT_AWAITING)
+MSG-OP-319: "Billing &lt;billing no&gt; was already sent" (DP_BILLING_SENT)
+MSG-OP-320: "Account &lt;invoice no&gt; is not confirmed for billing (&lt;tag&gt;)" (DP_ITEM_STATE)
+MSG-OP-321: "No account is confirmed for billing" (DP_NOTHING_TO_BILL)
+MSG-OP-322: "Invoice &lt;invoice no&gt; is not on billing &lt;billing no&gt;" (DP_NOT_ON_BILLING)
+MSG-OP-323: "Enter the e-mail address of &lt;insurer code&gt;" (DP_NO_RECIPIENT)
+MSG-OP-324: "Give the insurer's reason for rejecting &lt;invoice no&gt;" (DP_REASON_REQUIRED)
+MSG-OP-325: "Choose a direct payment reinstatement reason" (DP_REINSTATE_REASON)
+MSG-OP-326: "Invoice &lt;invoice no&gt; is not tagged direct payment by Marketing: its premium receivable cannot be reversed" (DP_TAG_INVALID)</t>
         </is>
       </c>
       <c r="M384" s="12" t="inlineStr">
@@ -42433,9 +42434,9 @@
       <c r="L385" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-328: "Billing &lt;billing no&gt; does not exist" (DP_BILLING_UNKNOWN)
-MSG-OP-329: "Decision '&lt;decision&gt;' is not one of Approved or Rejected (or Yes / No)" (DP_RESPONSE_DECISION)
-MSG-OP-330: "The insurer's answer has no '&lt;header&gt;' column" (DP_RESPONSE_LAYOUT)</t>
+MSG-OP-329: "Billing &lt;billing no&gt; does not exist" (DP_BILLING_UNKNOWN)
+MSG-OP-330: "Decision '&lt;decision&gt;' is not one of Approved or Rejected (or Yes / No)" (DP_RESPONSE_DECISION)
+MSG-OP-331: "The insurer's answer has no '&lt;header&gt;' column" (DP_RESPONSE_LAYOUT)</t>
         </is>
       </c>
       <c r="M385" s="12" t="inlineStr">
@@ -42510,10 +42511,10 @@
       <c r="L386" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-333: "Incentive scheme already exists: &lt;key&gt;" (DUPLICATE)
-MSG-OP-334: "The scheme ends before it starts" (INCENTIVE_SCHEME_DATES)
-MSG-OP-335: "Each tier needs a minimum basic premium and a fixed amount above zero" (INCENTIVE_TIER_INVALID)
-MSG-OP-336: "Each tier needs a production target and a rate above zero" (INCENTIVE_TIER_INVALID)</t>
+MSG-OP-334: "Incentive scheme already exists: &lt;key&gt;" (DUPLICATE)
+MSG-OP-335: "The scheme ends before it starts" (INCENTIVE_SCHEME_DATES)
+MSG-OP-336: "Each tier needs a minimum basic premium and a fixed amount above zero" (INCENTIVE_TIER_INVALID)
+MSG-OP-337: "Each tier needs a production target and a rate above zero" (INCENTIVE_TIER_INVALID)</t>
         </is>
       </c>
       <c r="M386" s="12" t="inlineStr">
@@ -42588,11 +42589,11 @@
       <c r="L387" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-338: "The company has no head office branch" (INCENTIVE_NO_HEAD_OFFICE)
-MSG-OP-339: "Run &lt;run no&gt; earned no incentive to post" (INCENTIVE_RUN_NOTHING)
-MSG-OP-340: "The period ends before it starts" (INCENTIVE_RUN_PERIOD)
-MSG-OP-341: "Run &lt;run no&gt; is &lt;status&gt; and cannot change" (INCENTIVE_RUN_STATE)
-MSG-OP-342: "Scheme &lt;name&gt; has no tiers yet: add its targets and amounts first" (INCENTIVE_SCHEME_EMPTY)</t>
+MSG-OP-339: "The company has no head office branch" (INCENTIVE_NO_HEAD_OFFICE)
+MSG-OP-340: "Run &lt;run no&gt; earned no incentive to post" (INCENTIVE_RUN_NOTHING)
+MSG-OP-341: "The period ends before it starts" (INCENTIVE_RUN_PERIOD)
+MSG-OP-342: "Run &lt;run no&gt; is &lt;status&gt; and cannot change" (INCENTIVE_RUN_STATE)
+MSG-OP-343: "Scheme &lt;name&gt; has no tiers yet: add its targets and amounts first" (INCENTIVE_SCHEME_EMPTY)</t>
         </is>
       </c>
       <c r="M387" s="12" t="inlineStr">
@@ -42667,12 +42668,12 @@
       <c r="L388" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-345: "The tax withheld must be above zero" (CERT_AMOUNT)
-MSG-OP-346: "Choose the company and the insurer of the certificate" (CERT_INSURER_REQUIRED)
-MSG-OP-347: "Only a rejected submission can be resubmitted" (CERT_NOT_REJECTED)
-MSG-OP-348: "Tag the certificate to at least one official receipt" (CERT_NO_OR)
-MSG-OP-349: "The certificate period ends before it starts" (CERT_PERIOD)
-MSG-OP-350: "Give the reason of the rejection" (CERT_REASON_REQUIRED)</t>
+MSG-OP-346: "The tax withheld must be above zero" (CERT_AMOUNT)
+MSG-OP-347: "Choose the company and the insurer of the certificate" (CERT_INSURER_REQUIRED)
+MSG-OP-348: "Only a rejected submission can be resubmitted" (CERT_NOT_REJECTED)
+MSG-OP-349: "Tag the certificate to at least one official receipt" (CERT_NO_OR)
+MSG-OP-350: "The certificate period ends before it starts" (CERT_PERIOD)
+MSG-OP-351: "Give the reason of the rejection" (CERT_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M388" s="12" t="inlineStr">
@@ -42747,12 +42748,12 @@
       <c r="L389" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-352: "An active scheme needs at least one tier"
-MSG-OP-353: "Enter a period that ends after it starts"
-MSG-OP-354: "Record the insurer decision of at least one account"
-MSG-OP-355: "The scheme ends before it starts"
-MSG-OP-356: "The scheme name is required"
-MSG-OP-357: "The tax withheld must be above zero"</t>
+MSG-OP-353: "An active scheme needs at least one tier"
+MSG-OP-354: "Enter a period that ends after it starts"
+MSG-OP-355: "Record the insurer decision of at least one account"
+MSG-OP-356: "The scheme ends before it starts"
+MSG-OP-357: "The scheme name is required"
+MSG-OP-358: "The tax withheld must be above zero"</t>
         </is>
       </c>
       <c r="M389" s="12" t="inlineStr">
@@ -42827,8 +42828,8 @@
       <c r="L390" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-361: "Feed &lt;code&gt; is inactive" (FLOW_IN_FEED_INACTIVE)
-MSG-OP-362: "No module processes uploads of feed &lt;feed code&gt; yet" (FLOW_IN_NO_HANDLER)</t>
+MSG-OP-362: "Feed &lt;code&gt; is inactive" (FLOW_IN_FEED_INACTIVE)
+MSG-OP-363: "No module processes uploads of feed &lt;feed code&gt; yet" (FLOW_IN_NO_HANDLER)</t>
         </is>
       </c>
       <c r="M390" s="12" t="inlineStr">
@@ -42891,9 +42892,9 @@
       <c r="L391" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-364: "Prefix is required"
-MSG-OP-366: "The range must end at or after its start"
-MSG-OP-367: "The series becomes active for issuing receipts."</t>
+MSG-OP-365: "Prefix is required"
+MSG-OP-367: "The range must end at or after its start"
+MSG-OP-368: "The series becomes active for issuing receipts."</t>
         </is>
       </c>
       <c r="M391" s="12" t="inlineStr">
@@ -42956,8 +42957,8 @@
       <c r="L392" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-368: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-OP-369: "&lt;Column&gt; is mandatory"</t>
+MSG-OP-369: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-OP-370: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M392" s="12" t="inlineStr">
@@ -43020,8 +43021,8 @@
       <c r="L393" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-370: "A certificate tag needs the certificate number"
-MSG-OP-371: "Path must be CASH or CERTIFICATE"</t>
+MSG-OP-371: "A certificate tag needs the certificate number"
+MSG-OP-372: "Path must be CASH or CERTIFICATE"</t>
         </is>
       </c>
       <c r="M393" s="12" t="inlineStr">
@@ -43084,7 +43085,7 @@
       <c r="L394" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-372: "Possible duplicate of &lt;preview&gt;"</t>
+MSG-OP-373: "Possible duplicate of &lt;preview&gt;"</t>
         </is>
       </c>
       <c r="M394" s="12" t="inlineStr">
@@ -43147,7 +43148,7 @@
       <c r="L395" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-373: "The amount must be above zero"</t>
+MSG-OP-374: "The amount must be above zero"</t>
         </is>
       </c>
       <c r="M395" s="12" t="inlineStr">
@@ -43210,7 +43211,7 @@
       <c r="L396" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-374: "The basic commission must be above zero"</t>
+MSG-OP-375: "The basic commission must be above zero"</t>
         </is>
       </c>
       <c r="M396" s="12" t="inlineStr">
@@ -43273,13 +43274,13 @@
       <c r="L397" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-OP-375: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-OP-376: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-OP-377: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-OP-378: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-OP-379: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-OP-380: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-OP-381: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-OP-376: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-OP-377: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-OP-378: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-OP-379: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-OP-380: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-OP-381: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-OP-382: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M397" s="12" t="inlineStr">

</xml_diff>